<commit_message>
Fix all 91 official property websites, Apartments.com listing URLs, and Show All Pins two-way toggle
</commit_message>
<xml_diff>
--- a/San_Jose_Apartments_Tracker.xlsx
+++ b/San_Jose_Apartments_Tracker.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="All Apartments (30)" sheetId="1" r:id="rId1"/>
+    <sheet name="All Apartments (91)" sheetId="1" r:id="rId1"/>
     <sheet name="Top Picks &amp; Sub-$3000" sheetId="2" r:id="rId2"/>
     <sheet name="Santa Clara SVP Zone" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -102,7 +102,7 @@
     <col min="17" max="20" width="13" customWidth="1"/>
     <col min="21" max="21" width="28" customWidth="1"/>
     <col min="22" max="23" width="46" customWidth="1"/>
-    <col min="24" max="25" width="36" customWidth="1"/>
+    <col min="24" max="26" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -228,6 +228,11 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Apartments.com Listing</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Official Website</t>
         </is>
       </c>
@@ -337,6 +342,11 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/north-park-apartment-homes-san-jose-ca/fsbvjbs/</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/san-jose/north-park.html</t>
         </is>
       </c>
@@ -446,6 +456,11 @@
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/crescent-village-apartment-homes-san-jose-ca/kb57kc8/</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/san-jose/crescent-village.html</t>
         </is>
       </c>
@@ -555,6 +570,11 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/enso-san-jose-ca/e5b3e4m/</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/enso</t>
         </is>
       </c>
@@ -664,7 +684,12 @@
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>https://www.aireliving.com/</t>
+          <t>https://www.apartments.com/aire-san-jose-ca/nrsnnzq/</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>https://aireliving.com/</t>
         </is>
       </c>
     </row>
@@ -775,7 +800,12 @@
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>https://www.fairfieldresidential.com/property/the-verdant-apartments/</t>
+          <t>https://www.apartments.com/the-verdant-apartments-san-jose-ca/9bng3w5/</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.fairfieldresidential.com/apartments/ca/san-jose/the-verdant-apartments/</t>
         </is>
       </c>
     </row>
@@ -884,6 +914,11 @@
       </c>
       <c r="Y7" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/epic-san-jose-ca/l8r08lg/</t>
+        </is>
+      </c>
+      <c r="Z7" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/epic</t>
         </is>
       </c>
@@ -993,6 +1028,11 @@
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/elan-at-river-oaks-san-jose-ca/9mqqy17/</t>
+        </is>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
           <t>https://www.sheaapartments.com/apartments/elan-at-river-oaks/</t>
         </is>
       </c>
@@ -1102,6 +1142,11 @@
       </c>
       <c r="Y9" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/river-view-apartment-homes-san-jose-ca/3hg41rd/</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/san-jose/river-view.html</t>
         </is>
       </c>
@@ -1213,7 +1258,12 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/vista-99-san-jose-ca/w00sz1l/</t>
+          <t>https://www.apartments.com/vista-99-san-jose-ca/2vres89/</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.equityapartments.com/san-francisco-bay/north-san-jose/vista-99-apartments</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1372,12 @@
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com</t>
+          <t>https://www.apartments.com/passero-santa-clara-ca/vbeyz4d/</t>
+        </is>
+      </c>
+      <c r="Z11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livepassero.com/</t>
         </is>
       </c>
     </row>
@@ -1433,7 +1488,12 @@
       </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>https://www.equityapartments.com/san-francisco-bay-area/santa-clara/estancia-at-santa-clara-apartments</t>
+          <t>https://www.apartments.com/estancia-at-santa-clara-santa-clara-ca/bfd2x09/</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/estancia-at-santa-clara-apartments</t>
         </is>
       </c>
     </row>
@@ -1544,6 +1604,11 @@
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/river-terrace-santa-clara-ca/dcr4v1l/</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
           <t>https://www.udr.com/san-francisco-bay-area-apartments/santa-clara/river-terrace/</t>
         </is>
       </c>
@@ -1655,7 +1720,12 @@
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>https://www.liveprado.com</t>
+          <t>https://www.apartments.com/prado-santa-clara-ca/b8re69b/</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liveprado.com/</t>
         </is>
       </c>
     </row>
@@ -1766,7 +1836,12 @@
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
-          <t>https://www.villasontheboulevard.com</t>
+          <t>https://www.apartments.com/villas-on-the-boulevard-santa-clara-ca/xpzkmpn/</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.villasontheboulevard.com/</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1952,12 @@
       </c>
       <c r="Y16" s="4" t="inlineStr">
         <is>
-          <t>https://www.prometheusapartments.com/santa-clara-ca/mansion-grove/</t>
+          <t>https://www.apartments.com/mansion-grove-santa-clara-ca/l36cb4f/</t>
+        </is>
+      </c>
+      <c r="Z16" s="4" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/mansion-grove/</t>
         </is>
       </c>
     </row>
@@ -1986,7 +2066,12 @@
       </c>
       <c r="Y17" s="3" t="inlineStr">
         <is>
-          <t>https://www.antonaspire.com</t>
+          <t>https://www.apartments.com/anton-aspire-milpitas-ca/ptmtmtt/</t>
+        </is>
+      </c>
+      <c r="Z17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.antonaspire.com/</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2180,12 @@
       </c>
       <c r="Y18" s="3" t="inlineStr">
         <is>
-          <t>https://www.centriaowners.com</t>
+          <t>https://www.apartments.com/centria-milpitas-ca/bvj0p49/</t>
+        </is>
+      </c>
+      <c r="Z18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.centriaowners.com/</t>
         </is>
       </c>
     </row>
@@ -2204,6 +2294,11 @@
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/apex-milpitas-ca/4vnellh/</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/milpitas/apex</t>
         </is>
       </c>
@@ -2315,7 +2410,12 @@
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>https://www.milpitascrossing.com</t>
+          <t>https://www.apartments.com/the-crossing-at-montague-milpitas-ca/843fym2/</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-crossing-at-montague-milpitas-ca/843fym2/</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2526,12 @@
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>https://www.amalfimilpitas.com</t>
+          <t>https://www.apartments.com/amalfi-apartments-milpitas-ca/yy8dzlr/</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>https://amalfimilpitas.com/</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2640,12 @@
       </c>
       <c r="Y22" s="2" t="inlineStr">
         <is>
-          <t>https://www.livethefields.com/turing</t>
+          <t>https://www.apartments.com/turing-at-the-fields-milpitas-ca/hx52vm1/</t>
+        </is>
+      </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thefieldsmilpitas.com/turing</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2754,12 @@
       </c>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>https://sheaproperties.com/apartments/northern-california/sixth-jackson-apartments/</t>
+          <t>https://www.apartments.com/sixth-jackson-san-jose-ca/xkhk1xp/</t>
+        </is>
+      </c>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sheaapartments.com/apartments/sixth-jackson/</t>
         </is>
       </c>
     </row>
@@ -2753,6 +2868,11 @@
       </c>
       <c r="Y24" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-esplanade-san-jose-ca/fb0vy0r/</t>
+        </is>
+      </c>
+      <c r="Z24" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/the-esplanade</t>
         </is>
       </c>
@@ -2862,6 +2982,11 @@
       </c>
       <c r="Y25" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-julian-san-jose-ca/few059v/</t>
+        </is>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
           <t>https://livethejulian.com/</t>
         </is>
       </c>
@@ -2971,7 +3096,12 @@
       </c>
       <c r="Y26" s="2" t="inlineStr">
         <is>
-          <t>https://www.essexapartmenthomes.com/apartments/san-jose/one-south-market</t>
+          <t>https://www.apartments.com/one-south-market-san-jose-ca/byxczjc/</t>
+        </is>
+      </c>
+      <c r="Z26" s="2" t="inlineStr">
+        <is>
+          <t>https://onesouthmarket.com/</t>
         </is>
       </c>
     </row>
@@ -3080,6 +3210,11 @@
       </c>
       <c r="Y27" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/marquis-san-jose-ca/qksmzqz/</t>
+        </is>
+      </c>
+      <c r="Z27" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/marquis</t>
         </is>
       </c>
@@ -3189,6 +3324,11 @@
       </c>
       <c r="Y28" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/patina-at-midtown-san-jose-ca/dxd0spl/</t>
+        </is>
+      </c>
+      <c r="Z28" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/patina-at-midtown</t>
         </is>
       </c>
@@ -3300,6 +3440,11 @@
       </c>
       <c r="Y29" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/avalon-on-the-alameda-san-jose-ca/pry6zvt/</t>
+        </is>
+      </c>
+      <c r="Z29" s="3" t="inlineStr">
+        <is>
           <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-on-the-alameda/</t>
         </is>
       </c>
@@ -3411,7 +3556,12 @@
       </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>https://www.livelynhaven.com/</t>
+          <t>https://www.apartments.com/lynhaven-san-jose-ca/tb0b949/</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>https://livelynhaven.com/</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3670,12 @@
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>https://www.vespaio.com/</t>
+          <t>https://www.apartments.com/vespaio-san-jose-ca/edr7h7p/</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.millcreekplaces.com/community/vespaio/</t>
         </is>
       </c>
     </row>
@@ -3532,7 +3687,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Viridian Apartments</t>
+          <t>Domain Apartments</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -3609,7 +3764,7 @@
       </c>
       <c r="U32" s="3" t="inlineStr">
         <is>
-          <t>Greystar / Institutional (Verified Institutional Community)</t>
+          <t>Greystar / Domain SJ (Verified Institutional Community)</t>
         </is>
       </c>
       <c r="V32" s="3" t="inlineStr">
@@ -3624,12 +3779,17 @@
       </c>
       <c r="X32" s="3" t="inlineStr">
         <is>
-          <t>3233 Zanker Rd, San Jose, CA 95134</t>
+          <t>1 Vista Montana, San Jose, CA 95134</t>
         </is>
       </c>
       <c r="Y32" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/san-jose-ca/</t>
+          <t>https://www.apartments.com/domain-apartments-san-jose-ca/k9lksnc/</t>
+        </is>
+      </c>
+      <c r="Z32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.domainsanjose.com/</t>
         </is>
       </c>
     </row>
@@ -3641,7 +3801,7 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Cerano Apartments</t>
+          <t>Willow Lake Apartment Homes</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -3718,7 +3878,7 @@
       </c>
       <c r="U33" s="3" t="inlineStr">
         <is>
-          <t>Shea Properties (Verified Institutional Developer (Shea))</t>
+          <t>Essex Property Trust (Verified Institutional Developer (Shea))</t>
         </is>
       </c>
       <c r="V33" s="3" t="inlineStr">
@@ -3733,12 +3893,17 @@
       </c>
       <c r="X33" s="3" t="inlineStr">
         <is>
-          <t>575 E Brokaw Rd, San Jose, CA 95112</t>
+          <t>1331 Lakeshore Cir, San Jose, CA 95131</t>
         </is>
       </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
-          <t>https://www.sheaapartments.com/apartments/cerano/</t>
+          <t>https://www.apartments.com/willow-lake-san-jose-ca/1yxldw7/</t>
+        </is>
+      </c>
+      <c r="Z33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/san-jose/willow-lake</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3915,7 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Corsa at Market Park (Berryessa BART)</t>
+          <t>Woodland Meadow Apartments</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -3827,7 +3992,7 @@
       </c>
       <c r="U34" s="2" t="inlineStr">
         <is>
-          <t>Greystar (Verified New-Build Transit Village (2021+))</t>
+          <t>Woodmont Real Estate Services (Verified New-Build Transit Village (2021+))</t>
         </is>
       </c>
       <c r="V34" s="2" t="inlineStr">
@@ -3842,12 +4007,17 @@
       </c>
       <c r="X34" s="2" t="inlineStr">
         <is>
-          <t>1550 Berryessa Rd, San Jose, CA 95133</t>
+          <t>1600 Whitewood Dr, San Jose, CA 95131</t>
         </is>
       </c>
       <c r="Y34" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/san-jose-ca/</t>
+          <t>https://www.apartments.com/woodland-meadow-san-jose-ca/v3y9hzd/</t>
+        </is>
+      </c>
+      <c r="Z34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.woodlandmeadow.com/apartments/ca/san-jose/floor-plans</t>
         </is>
       </c>
     </row>
@@ -3956,6 +4126,11 @@
       </c>
       <c r="Y35" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/santa-clara-square-apartment-homes-santa-clara-ca/rqgtnx3/</t>
+        </is>
+      </c>
+      <c r="Z35" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/santa-clara/santa-clara-square.html</t>
         </is>
       </c>
@@ -3968,7 +4143,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Riva Terra Apartments</t>
+          <t>Bella Vista Apartments</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -4047,7 +4222,7 @@
       </c>
       <c r="U36" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Institutional Community)</t>
+          <t>Interstate Equities / Bella Vista (Verified Institutional Community)</t>
         </is>
       </c>
       <c r="V36" s="3" t="inlineStr">
@@ -4062,12 +4237,17 @@
       </c>
       <c r="X36" s="3" t="inlineStr">
         <is>
-          <t>2900 Lakeside Dr, Santa Clara, CA 95054</t>
+          <t>1500 Vista Club Cir, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y36" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/riva-terra-santa-clara-ca/65k9eeu/</t>
+          <t>https://www.apartments.com/bella-vista-santa-clara-ca/lc3w7ng/</t>
+        </is>
+      </c>
+      <c r="Z36" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bellavista-apartments.com/</t>
         </is>
       </c>
     </row>
@@ -4079,7 +4259,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Station 1 (Lawrence Station)</t>
+          <t>Marina Cove Apartment Homes</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -4156,7 +4336,7 @@
       </c>
       <c r="U37" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Transit-Oriented Community)</t>
+          <t>Essex Property Trust (Verified Transit-Oriented Community)</t>
         </is>
       </c>
       <c r="V37" s="3" t="inlineStr">
@@ -4171,12 +4351,17 @@
       </c>
       <c r="X37" s="3" t="inlineStr">
         <is>
-          <t>3515 Reed Ave, Santa Clara, CA 95051</t>
+          <t>3480 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y37" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/santa-clara-ca/</t>
+          <t>https://www.apartments.com/marina-cove-santa-clara-ca/gsl8bkx/</t>
+        </is>
+      </c>
+      <c r="Z37" s="3" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/santa-clara/marina-cove</t>
         </is>
       </c>
     </row>
@@ -4285,6 +4470,11 @@
       </c>
       <c r="Y38" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/avalon-silicon-valley-sunnyvale-ca/we0jcgj/</t>
+        </is>
+      </c>
+      <c r="Z38" s="3" t="inlineStr">
+        <is>
           <t>https://www.avaloncommunities.com/california/sunnyvale-apartments/avalon-silicon-valley/</t>
         </is>
       </c>
@@ -4374,7 +4564,7 @@
       </c>
       <c r="U39" s="2" t="inlineStr">
         <is>
-          <t>Prometheus Real Estate Group (Verified Regional Operator (Prometheus))</t>
+          <t>Essex Property Trust (Verified Regional Operator (Prometheus))</t>
         </is>
       </c>
       <c r="V39" s="2" t="inlineStr">
@@ -4394,7 +4584,12 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/solstice/</t>
+          <t>https://www.apartments.com/solstice-sunnyvale-ca/5y4elen/</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/solstice</t>
         </is>
       </c>
     </row>
@@ -4503,7 +4698,12 @@
       </c>
       <c r="Y40" s="2" t="inlineStr">
         <is>
-          <t>https://www.centerrasj.com/</t>
+          <t>https://www.apartments.com/centerra-san-jose-ca/fs8gvdr/</t>
+        </is>
+      </c>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>https://liveatcenterra.com/</t>
         </is>
       </c>
     </row>
@@ -4612,7 +4812,12 @@
       </c>
       <c r="Y41" s="2" t="inlineStr">
         <is>
-          <t>https://www.millcreekplaces.com/community/modera-san-pedro-square/</t>
+          <t>https://www.apartments.com/modera-san-pedro-square-san-jose-ca/5m60lvp/</t>
+        </is>
+      </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.moderasanpedrosquare.com/</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4926,12 @@
       </c>
       <c r="Y42" s="2" t="inlineStr">
         <is>
-          <t>https://mirosanjose.com/</t>
+          <t>https://www.apartments.com/miro-san-jose-ca/bsvyvv8/</t>
+        </is>
+      </c>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rentmiro.com/</t>
         </is>
       </c>
     </row>
@@ -4830,6 +5040,11 @@
       </c>
       <c r="Y43" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/121-tasman-san-jose-ca/pdbxmnt/</t>
+        </is>
+      </c>
+      <c r="Z43" s="2" t="inlineStr">
+        <is>
           <t>https://www.121tasman.com/</t>
         </is>
       </c>
@@ -4939,6 +5154,11 @@
       </c>
       <c r="Y44" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/venue-apartments-san-jose-ca/vkhxjjd/</t>
+        </is>
+      </c>
+      <c r="Z44" s="3" t="inlineStr">
+        <is>
           <t>https://www.venue-apts.com/</t>
         </is>
       </c>
@@ -5048,6 +5268,11 @@
       </c>
       <c r="Y45" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/1036-onofrio-ln-san-jose-ca/zz84sdz/</t>
+        </is>
+      </c>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
           <t>https://www.theplatformapts.com/</t>
         </is>
       </c>
@@ -5157,7 +5382,12 @@
       </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
-          <t>https://www.liveatlinq.com/</t>
+          <t>https://www.apartments.com/linq-san-jose-ca/d325jkj/</t>
+        </is>
+      </c>
+      <c r="Z46" s="3" t="inlineStr">
+        <is>
+          <t>https://liveatlinq.com/</t>
         </is>
       </c>
     </row>
@@ -5268,6 +5498,11 @@
       </c>
       <c r="Y47" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/sofi-berryessa-san-jose-ca/pnhhkct/</t>
+        </is>
+      </c>
+      <c r="Z47" s="2" t="inlineStr">
+        <is>
           <t>https://www.sofiberryessa.com/</t>
         </is>
       </c>
@@ -5377,7 +5612,12 @@
       </c>
       <c r="Y48" s="2" t="inlineStr">
         <is>
-          <t>https://griffisresidential.com/apartments/ca/milpitas/griffis-south-bay/</t>
+          <t>https://www.apartments.com/griffis-south-bay-milpitas-ca/8qvze43/</t>
+        </is>
+      </c>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>https://griffisresidential.com/property/south-bay/</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5728,12 @@
       </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
-          <t>https://www.edgemilpitas.com/</t>
+          <t>https://www.apartments.com/the-edge-milpitas-ca/rn2vmg3/</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
+          <t>https://edgemilpitas.com/</t>
         </is>
       </c>
     </row>
@@ -5599,6 +5844,11 @@
       </c>
       <c r="Y50" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/312-gates-dr-milpitas-ca-unit-si-fl2-id2002/r9hml32/</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
           <t>https://www.exploreeleanor.com/</t>
         </is>
       </c>
@@ -5708,6 +5958,11 @@
       </c>
       <c r="Y51" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-harlowe-milpitas-ca/ygpz47v/</t>
+        </is>
+      </c>
+      <c r="Z51" s="3" t="inlineStr">
+        <is>
           <t>https://www.harloweliving.com/</t>
         </is>
       </c>
@@ -5819,7 +6074,12 @@
       </c>
       <c r="Y52" s="2" t="inlineStr">
         <is>
-          <t>https://www.lantanamilpitas.com/</t>
+          <t>https://www.apartments.com/lantana-at-milpitas-station-milpitas-ca/2gq4v3c/</t>
+        </is>
+      </c>
+      <c r="Z52" s="2" t="inlineStr">
+        <is>
+          <t>https://lantanamilpitas.com/</t>
         </is>
       </c>
     </row>
@@ -5928,6 +6188,11 @@
       </c>
       <c r="Y53" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/ilara-milpitas-ca/cz269te/</t>
+        </is>
+      </c>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
           <t>https://www.ilaraapartments.com/</t>
         </is>
       </c>
@@ -6039,6 +6304,11 @@
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/mill-creek-milpitas-ca/vm1tzld/</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/milpitas/mill-creek-apartments</t>
         </is>
       </c>
@@ -6150,7 +6420,12 @@
       </c>
       <c r="Y55" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/milpitas-ca/</t>
+          <t>https://www.apartments.com/parc-west-milpitas-ca/sbe86w7/</t>
+        </is>
+      </c>
+      <c r="Z55" s="2" t="inlineStr">
+        <is>
+          <t>https://www.themuirfieldcompany.com/properties</t>
         </is>
       </c>
     </row>
@@ -6261,7 +6536,12 @@
       </c>
       <c r="Y56" s="3" t="inlineStr">
         <is>
-          <t>https://www.sheaapartments.com/</t>
+          <t>https://www.apartments.com/building/terra-serena-luna-milpitas-ca/rws26s0/</t>
+        </is>
+      </c>
+      <c r="Z56" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/building/terra-serena-luna-milpitas-ca/rws26s0/</t>
         </is>
       </c>
     </row>
@@ -6370,7 +6650,12 @@
       </c>
       <c r="Y57" s="3" t="inlineStr">
         <is>
-          <t>https://www.550moreland.com/</t>
+          <t>https://www.apartments.com/550-moreland-santa-clara-ca/ypyh9ns/</t>
+        </is>
+      </c>
+      <c r="Z57" s="3" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/550-moreland</t>
         </is>
       </c>
     </row>
@@ -6479,7 +6764,12 @@
       </c>
       <c r="Y58" s="3" t="inlineStr">
         <is>
-          <t>https://www.aveliving.com/locations/san-francisco-bay-area/santa-clara/ave-santa-clara</t>
+          <t>https://www.apartments.com/ave-santa-clara-santa-clara-ca/z3k89nx/</t>
+        </is>
+      </c>
+      <c r="Z58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aveliving.com/locations/south-bay-silicon-valley/santa-clara</t>
         </is>
       </c>
     </row>
@@ -6588,7 +6878,12 @@
       </c>
       <c r="Y59" s="3" t="inlineStr">
         <is>
-          <t>https://www.thelafayettesantaclara.com/</t>
+          <t>https://www.apartments.com/the-lafayette-santa-clara-ca/c3enymd/</t>
+        </is>
+      </c>
+      <c r="Z59" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livethelafayette.com/</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6992,12 @@
       </c>
       <c r="Y60" s="2" t="inlineStr">
         <is>
-          <t>https://www.theclaraapartments.com/</t>
+          <t>https://www.apartments.com/the-clara-santa-clara-ca/6b3v70v/</t>
+        </is>
+      </c>
+      <c r="Z60" s="2" t="inlineStr">
+        <is>
+          <t>https://theclara.com/</t>
         </is>
       </c>
     </row>
@@ -6808,6 +7108,11 @@
       </c>
       <c r="Y61" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/monticello-apartment-homes-santa-clara-ca/svq6gr4/</t>
+        </is>
+      </c>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/santa-clara/monticello.html</t>
         </is>
       </c>
@@ -6917,6 +7222,11 @@
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/mylo-santa-clara-santa-clara-ca/1rn76d4/</t>
+        </is>
+      </c>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/santa-clara/mylo-santa-clara</t>
         </is>
       </c>
@@ -7026,6 +7336,11 @@
       </c>
       <c r="Y63" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/lorien-santa-clara-ca/ls5tjef/</t>
+        </is>
+      </c>
+      <c r="Z63" s="3" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/lorien-apartments</t>
         </is>
       </c>
@@ -7137,7 +7452,12 @@
       </c>
       <c r="Y64" s="2" t="inlineStr">
         <is>
-          <t>https://www.deanzaproperties.com/apartments/ca/santa-clara/catalina-luxury-apartments/</t>
+          <t>https://www.apartments.com/catalina-luxury-apartments-santa-clara-ca/5d8x1hm/</t>
+        </is>
+      </c>
+      <c r="Z64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deanzaproperties.com/south-bay-area/catalina-luxury-apartments/</t>
         </is>
       </c>
     </row>
@@ -7248,6 +7568,11 @@
       </c>
       <c r="Y65" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/villa-granada-santa-clara-ca/q89dqzw/</t>
+        </is>
+      </c>
+      <c r="Z65" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/santa-clara/villa-granada</t>
         </is>
       </c>
@@ -7357,7 +7682,12 @@
       </c>
       <c r="Y66" s="2" t="inlineStr">
         <is>
-          <t>https://www.prometheusapartments.com/ca/santa-clara-apartments/cobalt</t>
+          <t>https://www.apartments.com/cobalt-santa-clara-ca/pnpkzps/</t>
+        </is>
+      </c>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/cobalt</t>
         </is>
       </c>
     </row>
@@ -7466,7 +7796,12 @@
       </c>
       <c r="Y67" s="3" t="inlineStr">
         <is>
-          <t>https://www.hollandresidential.com/ca/santa-clara/orlo</t>
+          <t>https://www.apartments.com/orlo-and-alba-santa-clara-ca/1pw4vv6/</t>
+        </is>
+      </c>
+      <c r="Z67" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hollandresidential.com/ca/santa-clara/orlo-alba</t>
         </is>
       </c>
     </row>
@@ -7575,6 +7910,11 @@
       </c>
       <c r="Y68" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/domicilio-santa-clara-ca/6x81pwt/</t>
+        </is>
+      </c>
+      <c r="Z68" s="3" t="inlineStr">
+        <is>
           <t>https://www.domicilioapts.com/</t>
         </is>
       </c>
@@ -7684,7 +8024,12 @@
       </c>
       <c r="Y69" s="3" t="inlineStr">
         <is>
-          <t>https://www.missionpointebywindsor.com/</t>
+          <t>https://www.apartments.com/mission-pointe-by-windsor-sunnyvale-ca/j83gb95/</t>
+        </is>
+      </c>
+      <c r="Z69" s="3" t="inlineStr">
+        <is>
+          <t>https://www.windsorcommunities.com/properties/mission-pointe-by-windsor/</t>
         </is>
       </c>
     </row>
@@ -7793,6 +8138,11 @@
       </c>
       <c r="Y70" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/encasa-sunnyvale-ca/s1ktnb6/</t>
+        </is>
+      </c>
+      <c r="Z70" s="2" t="inlineStr">
+        <is>
           <t>https://www.encasaliving.com/</t>
         </is>
       </c>
@@ -7904,6 +8254,11 @@
       </c>
       <c r="Y71" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-arches-sunnyvale-ca/fvycn0r/</t>
+        </is>
+      </c>
+      <c r="Z71" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/sunnyvale/the-arches-apartments</t>
         </is>
       </c>
@@ -8013,6 +8368,11 @@
       </c>
       <c r="Y72" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-montclaire-sunnyvale-ca/x4m85qp/</t>
+        </is>
+      </c>
+      <c r="Z72" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/the-montclaire</t>
         </is>
       </c>
@@ -8124,6 +8484,11 @@
       </c>
       <c r="Y73" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/windsor-ridge-sunnyvale-ca/nsgs57p/</t>
+        </is>
+      </c>
+      <c r="Z73" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/windsor-ridge</t>
         </is>
       </c>
@@ -8235,6 +8600,11 @@
       </c>
       <c r="Y74" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/briarwood-sunnyvale-ca/v07q4kg/</t>
+        </is>
+      </c>
+      <c r="Z74" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/sunnyvale/briarwood-apartments</t>
         </is>
       </c>
@@ -8344,7 +8714,12 @@
       </c>
       <c r="Y75" s="2" t="inlineStr">
         <is>
-          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/spruce/</t>
+          <t>https://www.apartments.com/spruce-apartments-sunnyvale-ca/prxrltv/</t>
+        </is>
+      </c>
+      <c r="Z75" s="2" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/spruce</t>
         </is>
       </c>
     </row>
@@ -8453,6 +8828,11 @@
       </c>
       <c r="Y76" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/arbor-terrace-sunnyvale-ca/z3qzypx/</t>
+        </is>
+      </c>
+      <c r="Z76" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/sunnyvale/arbor-terrace-apartments</t>
         </is>
       </c>
@@ -8564,6 +8944,11 @@
       </c>
       <c r="Y77" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/magnolia-square-sunnyvale-ca/zstdbqz/</t>
+        </is>
+      </c>
+      <c r="Z77" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/magnolia-square</t>
         </is>
       </c>
@@ -8675,7 +9060,12 @@
       </c>
       <c r="Y78" s="2" t="inlineStr">
         <is>
-          <t>https://www.windsorcommunities.com/properties/pavona/</t>
+          <t>https://www.apartments.com/pavona-apartments-san-jose-ca/qf6de5z/</t>
+        </is>
+      </c>
+      <c r="Z78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.windsorcommunities.com/properties/pavona-apartments/</t>
         </is>
       </c>
     </row>
@@ -8784,6 +9174,11 @@
       </c>
       <c r="Y79" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/cannery-park-by-windsor-san-jose-ca/43ekybk/</t>
+        </is>
+      </c>
+      <c r="Z79" s="3" t="inlineStr">
+        <is>
           <t>https://www.windsorcommunities.com/properties/cannery-park-by-windsor/</t>
         </is>
       </c>
@@ -8893,7 +9288,12 @@
       </c>
       <c r="Y80" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/villa-torino-san-jose-ca/</t>
+          <t>https://www.apartments.com/villa-torino-san-jose-ca/40372th/</t>
+        </is>
+      </c>
+      <c r="Z80" s="2" t="inlineStr">
+        <is>
+          <t>https://www.villatorinoapts.com/</t>
         </is>
       </c>
     </row>
@@ -9002,6 +9402,11 @@
       </c>
       <c r="Y81" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/360-residences-san-jose-ca/xx7h13n/</t>
+        </is>
+      </c>
+      <c r="Z81" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/360-residences</t>
         </is>
       </c>
@@ -9014,7 +9419,7 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>The Fay (SoFA Luxury Tower)</t>
+          <t>Flow San Jose (formerly The Fay)</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -9111,7 +9516,12 @@
       </c>
       <c r="Y82" s="3" t="inlineStr">
         <is>
-          <t>https://www.thefaysj.com/</t>
+          <t>https://www.apartments.com/flow-san-jose-san-jose-ca/12knvq5/</t>
+        </is>
+      </c>
+      <c r="Z82" s="3" t="inlineStr">
+        <is>
+          <t>https://flow.life/en/properties/san-jose</t>
         </is>
       </c>
     </row>
@@ -9220,6 +9630,11 @@
       </c>
       <c r="Y83" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-pierce-san-jose-ca/533ct9n/</t>
+        </is>
+      </c>
+      <c r="Z83" s="2" t="inlineStr">
+        <is>
           <t>https://www.thepierce.com/</t>
         </is>
       </c>
@@ -9324,12 +9739,17 @@
       </c>
       <c r="X84" s="3" t="inlineStr">
         <is>
-          <t>715 W Julian St, San Jose, CA 95126</t>
+          <t>717 W Julian St, San Jose, CA 95126</t>
         </is>
       </c>
       <c r="Y84" s="3" t="inlineStr">
         <is>
-          <t>https://www.diridonwest.com/</t>
+          <t>https://www.apartments.com/diridon-west-san-jose-ca/l194cvd/</t>
+        </is>
+      </c>
+      <c r="Z84" s="3" t="inlineStr">
+        <is>
+          <t>https://diridonwest.com/</t>
         </is>
       </c>
     </row>
@@ -9341,7 +9761,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Modera The Alameda</t>
+          <t>787 The Alameda (formerly Modera The Alameda)</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -9438,7 +9858,12 @@
       </c>
       <c r="Y85" s="3" t="inlineStr">
         <is>
-          <t>https://www.millcreekplaces.com/community/modera-the-alameda/</t>
+          <t>https://www.apartments.com/787-the-alameda-san-jose-ca/7f64s5w/</t>
+        </is>
+      </c>
+      <c r="Z85" s="3" t="inlineStr">
+        <is>
+          <t>https://www.787thealameda.com/</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9875,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Avalon Morrison Park</t>
+          <t>Bell Diridon (formerly Avalon Morrison Park)</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -9549,7 +9974,12 @@
       </c>
       <c r="Y86" s="3" t="inlineStr">
         <is>
-          <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-morrison-park/</t>
+          <t>https://www.apartments.com/bell-diridon-san-jose-ca/q9197cx/</t>
+        </is>
+      </c>
+      <c r="Z86" s="3" t="inlineStr">
+        <is>
+          <t>https://www.belldiridon.com/</t>
         </is>
       </c>
     </row>
@@ -9658,7 +10088,12 @@
       </c>
       <c r="Y87" s="2" t="inlineStr">
         <is>
-          <t>https://www.meridianmidtown.com/</t>
+          <t>https://www.apartments.com/meridian-at-midtown-san-jose-ca/ezyhf1m/</t>
+        </is>
+      </c>
+      <c r="Z87" s="2" t="inlineStr">
+        <is>
+          <t>https://meridianmidtown.com/</t>
         </is>
       </c>
     </row>
@@ -9769,7 +10204,12 @@
       </c>
       <c r="Y88" s="2" t="inlineStr">
         <is>
-          <t>https://www.elementsmidtown.com/</t>
+          <t>https://www.apartments.com/elements-san-jose-ca/v3ky8zd/</t>
+        </is>
+      </c>
+      <c r="Z88" s="2" t="inlineStr">
+        <is>
+          <t>https://www.elementsapts.com/</t>
         </is>
       </c>
     </row>
@@ -9878,6 +10318,11 @@
       </c>
       <c r="Y89" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/808-west-apartments-san-jose-ca/402fkjh/</t>
+        </is>
+      </c>
+      <c r="Z89" s="2" t="inlineStr">
+        <is>
           <t>https://www.808west-apts.com/</t>
         </is>
       </c>
@@ -9989,6 +10434,11 @@
       </c>
       <c r="Y90" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/embark-apartments-fremont-ca/c2hfn5g/</t>
+        </is>
+      </c>
+      <c r="Z90" s="3" t="inlineStr">
+        <is>
           <t>https://www.embarkapartments.com/</t>
         </is>
       </c>
@@ -10001,7 +10451,7 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Amara at Tasman East</t>
+          <t>Marina Playa Apartment Homes</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -10078,7 +10528,7 @@
       </c>
       <c r="U91" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Active Community (Greystar))</t>
+          <t>UDR (Verified Active Community (Greystar))</t>
         </is>
       </c>
       <c r="V91" s="3" t="inlineStr">
@@ -10093,12 +10543,17 @@
       </c>
       <c r="X91" s="3" t="inlineStr">
         <is>
-          <t>2233 Calle Del Mundo, Santa Clara, CA 95054</t>
+          <t>3500 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y91" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com/</t>
+          <t>https://www.apartments.com/marina-playa-santa-clara-ca/d6tg4dk/</t>
+        </is>
+      </c>
+      <c r="Z91" s="3" t="inlineStr">
+        <is>
+          <t>https://www.udr.com/san-francisco-bay-area-apartments/santa-clara/marina-playa/</t>
         </is>
       </c>
     </row>
@@ -10204,12 +10659,17 @@
       </c>
       <c r="X92" s="2" t="inlineStr">
         <is>
-          <t>2250 Monroe St, Santa Clara, CA 95050</t>
+          <t>4500 Carlyle Ct, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y92" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/the-carlyle-santa-clara-ca/</t>
+          <t>https://www.apartments.com/carlyle-santa-clara-ca/j7b5mj7/</t>
+        </is>
+      </c>
+      <c r="Z92" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thecarlyle-apartments.com/</t>
         </is>
       </c>
     </row>
@@ -10227,7 +10687,7 @@
     <col min="17" max="20" width="13" customWidth="1"/>
     <col min="21" max="21" width="28" customWidth="1"/>
     <col min="22" max="23" width="46" customWidth="1"/>
-    <col min="24" max="25" width="36" customWidth="1"/>
+    <col min="24" max="26" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -10353,6 +10813,11 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Apartments.com Listing</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Official Website</t>
         </is>
       </c>
@@ -10462,6 +10927,11 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/north-park-apartment-homes-san-jose-ca/fsbvjbs/</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/san-jose/north-park.html</t>
         </is>
       </c>
@@ -10571,6 +11041,11 @@
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/crescent-village-apartment-homes-san-jose-ca/kb57kc8/</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/san-jose/crescent-village.html</t>
         </is>
       </c>
@@ -10680,6 +11155,11 @@
       </c>
       <c r="Y4" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/enso-san-jose-ca/e5b3e4m/</t>
+        </is>
+      </c>
+      <c r="Z4" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/enso</t>
         </is>
       </c>
@@ -10789,7 +11269,12 @@
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>https://www.aireliving.com/</t>
+          <t>https://www.apartments.com/aire-san-jose-ca/nrsnnzq/</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>https://aireliving.com/</t>
         </is>
       </c>
     </row>
@@ -10898,7 +11383,12 @@
       </c>
       <c r="Y6" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com</t>
+          <t>https://www.apartments.com/passero-santa-clara-ca/vbeyz4d/</t>
+        </is>
+      </c>
+      <c r="Z6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livepassero.com/</t>
         </is>
       </c>
     </row>
@@ -11009,7 +11499,12 @@
       </c>
       <c r="Y7" s="3" t="inlineStr">
         <is>
-          <t>https://www.equityapartments.com/san-francisco-bay-area/santa-clara/estancia-at-santa-clara-apartments</t>
+          <t>https://www.apartments.com/estancia-at-santa-clara-santa-clara-ca/bfd2x09/</t>
+        </is>
+      </c>
+      <c r="Z7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/estancia-at-santa-clara-apartments</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11613,12 @@
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
-          <t>https://www.antonaspire.com</t>
+          <t>https://www.apartments.com/anton-aspire-milpitas-ca/ptmtmtt/</t>
+        </is>
+      </c>
+      <c r="Z8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.antonaspire.com/</t>
         </is>
       </c>
     </row>
@@ -11227,7 +11727,12 @@
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>https://www.centriaowners.com</t>
+          <t>https://www.apartments.com/centria-milpitas-ca/bvj0p49/</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.centriaowners.com/</t>
         </is>
       </c>
     </row>
@@ -11336,6 +11841,11 @@
       </c>
       <c r="Y10" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/apex-milpitas-ca/4vnellh/</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/milpitas/apex</t>
         </is>
       </c>
@@ -11447,7 +11957,12 @@
       </c>
       <c r="Y11" s="2" t="inlineStr">
         <is>
-          <t>https://www.milpitascrossing.com</t>
+          <t>https://www.apartments.com/the-crossing-at-montague-milpitas-ca/843fym2/</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-crossing-at-montague-milpitas-ca/843fym2/</t>
         </is>
       </c>
     </row>
@@ -11558,7 +12073,12 @@
       </c>
       <c r="Y12" s="2" t="inlineStr">
         <is>
-          <t>https://www.amalfimilpitas.com</t>
+          <t>https://www.apartments.com/amalfi-apartments-milpitas-ca/yy8dzlr/</t>
+        </is>
+      </c>
+      <c r="Z12" s="2" t="inlineStr">
+        <is>
+          <t>https://amalfimilpitas.com/</t>
         </is>
       </c>
     </row>
@@ -11667,7 +12187,12 @@
       </c>
       <c r="Y13" s="2" t="inlineStr">
         <is>
-          <t>https://www.livethefields.com/turing</t>
+          <t>https://www.apartments.com/turing-at-the-fields-milpitas-ca/hx52vm1/</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thefieldsmilpitas.com/turing</t>
         </is>
       </c>
     </row>
@@ -11776,7 +12301,12 @@
       </c>
       <c r="Y14" s="3" t="inlineStr">
         <is>
-          <t>https://sheaproperties.com/apartments/northern-california/sixth-jackson-apartments/</t>
+          <t>https://www.apartments.com/sixth-jackson-san-jose-ca/xkhk1xp/</t>
+        </is>
+      </c>
+      <c r="Z14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sheaapartments.com/apartments/sixth-jackson/</t>
         </is>
       </c>
     </row>
@@ -11885,6 +12415,11 @@
       </c>
       <c r="Y15" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-esplanade-san-jose-ca/fb0vy0r/</t>
+        </is>
+      </c>
+      <c r="Z15" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/the-esplanade</t>
         </is>
       </c>
@@ -11994,6 +12529,11 @@
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-julian-san-jose-ca/few059v/</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
           <t>https://livethejulian.com/</t>
         </is>
       </c>
@@ -12103,7 +12643,12 @@
       </c>
       <c r="Y17" s="2" t="inlineStr">
         <is>
-          <t>https://www.essexapartmenthomes.com/apartments/san-jose/one-south-market</t>
+          <t>https://www.apartments.com/one-south-market-san-jose-ca/byxczjc/</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>https://onesouthmarket.com/</t>
         </is>
       </c>
     </row>
@@ -12212,6 +12757,11 @@
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/marquis-san-jose-ca/qksmzqz/</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/marquis</t>
         </is>
       </c>
@@ -12321,6 +12871,11 @@
       </c>
       <c r="Y19" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/patina-at-midtown-san-jose-ca/dxd0spl/</t>
+        </is>
+      </c>
+      <c r="Z19" s="3" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/patina-at-midtown</t>
         </is>
       </c>
@@ -12432,6 +12987,11 @@
       </c>
       <c r="Y20" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/avalon-on-the-alameda-san-jose-ca/pry6zvt/</t>
+        </is>
+      </c>
+      <c r="Z20" s="3" t="inlineStr">
+        <is>
           <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-on-the-alameda/</t>
         </is>
       </c>
@@ -12541,7 +13101,12 @@
       </c>
       <c r="Y21" s="2" t="inlineStr">
         <is>
-          <t>https://www.vespaio.com/</t>
+          <t>https://www.apartments.com/vespaio-san-jose-ca/edr7h7p/</t>
+        </is>
+      </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.millcreekplaces.com/community/vespaio/</t>
         </is>
       </c>
     </row>
@@ -12553,7 +13118,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Viridian Apartments</t>
+          <t>Domain Apartments</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -12630,7 +13195,7 @@
       </c>
       <c r="U22" s="3" t="inlineStr">
         <is>
-          <t>Greystar / Institutional (Verified Institutional Community)</t>
+          <t>Greystar / Domain SJ (Verified Institutional Community)</t>
         </is>
       </c>
       <c r="V22" s="3" t="inlineStr">
@@ -12645,12 +13210,17 @@
       </c>
       <c r="X22" s="3" t="inlineStr">
         <is>
-          <t>3233 Zanker Rd, San Jose, CA 95134</t>
+          <t>1 Vista Montana, San Jose, CA 95134</t>
         </is>
       </c>
       <c r="Y22" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/san-jose-ca/</t>
+          <t>https://www.apartments.com/domain-apartments-san-jose-ca/k9lksnc/</t>
+        </is>
+      </c>
+      <c r="Z22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.domainsanjose.com/</t>
         </is>
       </c>
     </row>
@@ -12662,7 +13232,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Cerano Apartments</t>
+          <t>Willow Lake Apartment Homes</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -12739,7 +13309,7 @@
       </c>
       <c r="U23" s="3" t="inlineStr">
         <is>
-          <t>Shea Properties (Verified Institutional Developer (Shea))</t>
+          <t>Essex Property Trust (Verified Institutional Developer (Shea))</t>
         </is>
       </c>
       <c r="V23" s="3" t="inlineStr">
@@ -12754,12 +13324,17 @@
       </c>
       <c r="X23" s="3" t="inlineStr">
         <is>
-          <t>575 E Brokaw Rd, San Jose, CA 95112</t>
+          <t>1331 Lakeshore Cir, San Jose, CA 95131</t>
         </is>
       </c>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>https://www.sheaapartments.com/apartments/cerano/</t>
+          <t>https://www.apartments.com/willow-lake-san-jose-ca/1yxldw7/</t>
+        </is>
+      </c>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/san-jose/willow-lake</t>
         </is>
       </c>
     </row>
@@ -12771,7 +13346,7 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Corsa at Market Park (Berryessa BART)</t>
+          <t>Woodland Meadow Apartments</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -12848,7 +13423,7 @@
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>Greystar (Verified New-Build Transit Village (2021+))</t>
+          <t>Woodmont Real Estate Services (Verified New-Build Transit Village (2021+))</t>
         </is>
       </c>
       <c r="V24" s="2" t="inlineStr">
@@ -12863,12 +13438,17 @@
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>1550 Berryessa Rd, San Jose, CA 95133</t>
+          <t>1600 Whitewood Dr, San Jose, CA 95131</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/san-jose-ca/</t>
+          <t>https://www.apartments.com/woodland-meadow-san-jose-ca/v3y9hzd/</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.woodlandmeadow.com/apartments/ca/san-jose/floor-plans</t>
         </is>
       </c>
     </row>
@@ -12977,6 +13557,11 @@
       </c>
       <c r="Y25" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/santa-clara-square-apartment-homes-santa-clara-ca/rqgtnx3/</t>
+        </is>
+      </c>
+      <c r="Z25" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/santa-clara/santa-clara-square.html</t>
         </is>
       </c>
@@ -12989,7 +13574,7 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Riva Terra Apartments</t>
+          <t>Bella Vista Apartments</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
@@ -13068,7 +13653,7 @@
       </c>
       <c r="U26" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Institutional Community)</t>
+          <t>Interstate Equities / Bella Vista (Verified Institutional Community)</t>
         </is>
       </c>
       <c r="V26" s="3" t="inlineStr">
@@ -13083,12 +13668,17 @@
       </c>
       <c r="X26" s="3" t="inlineStr">
         <is>
-          <t>2900 Lakeside Dr, Santa Clara, CA 95054</t>
+          <t>1500 Vista Club Cir, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y26" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/riva-terra-santa-clara-ca/65k9eeu/</t>
+          <t>https://www.apartments.com/bella-vista-santa-clara-ca/lc3w7ng/</t>
+        </is>
+      </c>
+      <c r="Z26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bellavista-apartments.com/</t>
         </is>
       </c>
     </row>
@@ -13100,7 +13690,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Station 1 (Lawrence Station)</t>
+          <t>Marina Cove Apartment Homes</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -13177,7 +13767,7 @@
       </c>
       <c r="U27" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Transit-Oriented Community)</t>
+          <t>Essex Property Trust (Verified Transit-Oriented Community)</t>
         </is>
       </c>
       <c r="V27" s="3" t="inlineStr">
@@ -13192,12 +13782,17 @@
       </c>
       <c r="X27" s="3" t="inlineStr">
         <is>
-          <t>3515 Reed Ave, Santa Clara, CA 95051</t>
+          <t>3480 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y27" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/santa-clara-ca/</t>
+          <t>https://www.apartments.com/marina-cove-santa-clara-ca/gsl8bkx/</t>
+        </is>
+      </c>
+      <c r="Z27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/santa-clara/marina-cove</t>
         </is>
       </c>
     </row>
@@ -13306,6 +13901,11 @@
       </c>
       <c r="Y28" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/avalon-silicon-valley-sunnyvale-ca/we0jcgj/</t>
+        </is>
+      </c>
+      <c r="Z28" s="3" t="inlineStr">
+        <is>
           <t>https://www.avaloncommunities.com/california/sunnyvale-apartments/avalon-silicon-valley/</t>
         </is>
       </c>
@@ -13395,7 +13995,7 @@
       </c>
       <c r="U29" s="2" t="inlineStr">
         <is>
-          <t>Prometheus Real Estate Group (Verified Regional Operator (Prometheus))</t>
+          <t>Essex Property Trust (Verified Regional Operator (Prometheus))</t>
         </is>
       </c>
       <c r="V29" s="2" t="inlineStr">
@@ -13415,7 +14015,12 @@
       </c>
       <c r="Y29" s="2" t="inlineStr">
         <is>
-          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/solstice/</t>
+          <t>https://www.apartments.com/solstice-sunnyvale-ca/5y4elen/</t>
+        </is>
+      </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/solstice</t>
         </is>
       </c>
     </row>
@@ -13524,7 +14129,12 @@
       </c>
       <c r="Y30" s="2" t="inlineStr">
         <is>
-          <t>https://www.centerrasj.com/</t>
+          <t>https://www.apartments.com/centerra-san-jose-ca/fs8gvdr/</t>
+        </is>
+      </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>https://liveatcenterra.com/</t>
         </is>
       </c>
     </row>
@@ -13633,7 +14243,12 @@
       </c>
       <c r="Y31" s="2" t="inlineStr">
         <is>
-          <t>https://www.millcreekplaces.com/community/modera-san-pedro-square/</t>
+          <t>https://www.apartments.com/modera-san-pedro-square-san-jose-ca/5m60lvp/</t>
+        </is>
+      </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.moderasanpedrosquare.com/</t>
         </is>
       </c>
     </row>
@@ -13742,7 +14357,12 @@
       </c>
       <c r="Y32" s="2" t="inlineStr">
         <is>
-          <t>https://mirosanjose.com/</t>
+          <t>https://www.apartments.com/miro-san-jose-ca/bsvyvv8/</t>
+        </is>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.rentmiro.com/</t>
         </is>
       </c>
     </row>
@@ -13851,6 +14471,11 @@
       </c>
       <c r="Y33" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/venue-apartments-san-jose-ca/vkhxjjd/</t>
+        </is>
+      </c>
+      <c r="Z33" s="3" t="inlineStr">
+        <is>
           <t>https://www.venue-apts.com/</t>
         </is>
       </c>
@@ -13960,7 +14585,12 @@
       </c>
       <c r="Y34" s="3" t="inlineStr">
         <is>
-          <t>https://www.liveatlinq.com/</t>
+          <t>https://www.apartments.com/linq-san-jose-ca/d325jkj/</t>
+        </is>
+      </c>
+      <c r="Z34" s="3" t="inlineStr">
+        <is>
+          <t>https://liveatlinq.com/</t>
         </is>
       </c>
     </row>
@@ -14069,7 +14699,12 @@
       </c>
       <c r="Y35" s="2" t="inlineStr">
         <is>
-          <t>https://griffisresidential.com/apartments/ca/milpitas/griffis-south-bay/</t>
+          <t>https://www.apartments.com/griffis-south-bay-milpitas-ca/8qvze43/</t>
+        </is>
+      </c>
+      <c r="Z35" s="2" t="inlineStr">
+        <is>
+          <t>https://griffisresidential.com/property/south-bay/</t>
         </is>
       </c>
     </row>
@@ -14178,6 +14813,11 @@
       </c>
       <c r="Y36" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-harlowe-milpitas-ca/ygpz47v/</t>
+        </is>
+      </c>
+      <c r="Z36" s="3" t="inlineStr">
+        <is>
           <t>https://www.harloweliving.com/</t>
         </is>
       </c>
@@ -14287,6 +14927,11 @@
       </c>
       <c r="Y37" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/ilara-milpitas-ca/cz269te/</t>
+        </is>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
           <t>https://www.ilaraapartments.com/</t>
         </is>
       </c>
@@ -14398,6 +15043,11 @@
       </c>
       <c r="Y38" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/mill-creek-milpitas-ca/vm1tzld/</t>
+        </is>
+      </c>
+      <c r="Z38" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/milpitas/mill-creek-apartments</t>
         </is>
       </c>
@@ -14509,7 +15159,12 @@
       </c>
       <c r="Y39" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/milpitas-ca/</t>
+          <t>https://www.apartments.com/parc-west-milpitas-ca/sbe86w7/</t>
+        </is>
+      </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>https://www.themuirfieldcompany.com/properties</t>
         </is>
       </c>
     </row>
@@ -14620,7 +15275,12 @@
       </c>
       <c r="Y40" s="3" t="inlineStr">
         <is>
-          <t>https://www.sheaapartments.com/</t>
+          <t>https://www.apartments.com/building/terra-serena-luna-milpitas-ca/rws26s0/</t>
+        </is>
+      </c>
+      <c r="Z40" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/building/terra-serena-luna-milpitas-ca/rws26s0/</t>
         </is>
       </c>
     </row>
@@ -14729,7 +15389,12 @@
       </c>
       <c r="Y41" s="3" t="inlineStr">
         <is>
-          <t>https://www.550moreland.com/</t>
+          <t>https://www.apartments.com/550-moreland-santa-clara-ca/ypyh9ns/</t>
+        </is>
+      </c>
+      <c r="Z41" s="3" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/550-moreland</t>
         </is>
       </c>
     </row>
@@ -14838,7 +15503,12 @@
       </c>
       <c r="Y42" s="3" t="inlineStr">
         <is>
-          <t>https://www.aveliving.com/locations/san-francisco-bay-area/santa-clara/ave-santa-clara</t>
+          <t>https://www.apartments.com/ave-santa-clara-santa-clara-ca/z3k89nx/</t>
+        </is>
+      </c>
+      <c r="Z42" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aveliving.com/locations/south-bay-silicon-valley/santa-clara</t>
         </is>
       </c>
     </row>
@@ -14947,7 +15617,12 @@
       </c>
       <c r="Y43" s="3" t="inlineStr">
         <is>
-          <t>https://www.thelafayettesantaclara.com/</t>
+          <t>https://www.apartments.com/the-lafayette-santa-clara-ca/c3enymd/</t>
+        </is>
+      </c>
+      <c r="Z43" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livethelafayette.com/</t>
         </is>
       </c>
     </row>
@@ -15056,6 +15731,11 @@
       </c>
       <c r="Y44" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/mylo-santa-clara-santa-clara-ca/1rn76d4/</t>
+        </is>
+      </c>
+      <c r="Z44" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/santa-clara/mylo-santa-clara</t>
         </is>
       </c>
@@ -15165,6 +15845,11 @@
       </c>
       <c r="Y45" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/lorien-santa-clara-ca/ls5tjef/</t>
+        </is>
+      </c>
+      <c r="Z45" s="3" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/lorien-apartments</t>
         </is>
       </c>
@@ -15274,7 +15959,12 @@
       </c>
       <c r="Y46" s="3" t="inlineStr">
         <is>
-          <t>https://www.hollandresidential.com/ca/santa-clara/orlo</t>
+          <t>https://www.apartments.com/orlo-and-alba-santa-clara-ca/1pw4vv6/</t>
+        </is>
+      </c>
+      <c r="Z46" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hollandresidential.com/ca/santa-clara/orlo-alba</t>
         </is>
       </c>
     </row>
@@ -15383,6 +16073,11 @@
       </c>
       <c r="Y47" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/domicilio-santa-clara-ca/6x81pwt/</t>
+        </is>
+      </c>
+      <c r="Z47" s="3" t="inlineStr">
+        <is>
           <t>https://www.domicilioapts.com/</t>
         </is>
       </c>
@@ -15492,7 +16187,12 @@
       </c>
       <c r="Y48" s="3" t="inlineStr">
         <is>
-          <t>https://www.missionpointebywindsor.com/</t>
+          <t>https://www.apartments.com/mission-pointe-by-windsor-sunnyvale-ca/j83gb95/</t>
+        </is>
+      </c>
+      <c r="Z48" s="3" t="inlineStr">
+        <is>
+          <t>https://www.windsorcommunities.com/properties/mission-pointe-by-windsor/</t>
         </is>
       </c>
     </row>
@@ -15601,6 +16301,11 @@
       </c>
       <c r="Y49" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/the-montclaire-sunnyvale-ca/x4m85qp/</t>
+        </is>
+      </c>
+      <c r="Z49" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/sunnyvale/the-montclaire</t>
         </is>
       </c>
@@ -15710,7 +16415,12 @@
       </c>
       <c r="Y50" s="2" t="inlineStr">
         <is>
-          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/spruce/</t>
+          <t>https://www.apartments.com/spruce-apartments-sunnyvale-ca/prxrltv/</t>
+        </is>
+      </c>
+      <c r="Z50" s="2" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/sunnyvale-apartments/spruce</t>
         </is>
       </c>
     </row>
@@ -15819,6 +16529,11 @@
       </c>
       <c r="Y51" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/arbor-terrace-sunnyvale-ca/z3qzypx/</t>
+        </is>
+      </c>
+      <c r="Z51" s="2" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/sunnyvale/arbor-terrace-apartments</t>
         </is>
       </c>
@@ -15928,6 +16643,11 @@
       </c>
       <c r="Y52" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/cannery-park-by-windsor-san-jose-ca/43ekybk/</t>
+        </is>
+      </c>
+      <c r="Z52" s="3" t="inlineStr">
+        <is>
           <t>https://www.windsorcommunities.com/properties/cannery-park-by-windsor/</t>
         </is>
       </c>
@@ -16037,7 +16757,12 @@
       </c>
       <c r="Y53" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/villa-torino-san-jose-ca/</t>
+          <t>https://www.apartments.com/villa-torino-san-jose-ca/40372th/</t>
+        </is>
+      </c>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>https://www.villatorinoapts.com/</t>
         </is>
       </c>
     </row>
@@ -16146,6 +16871,11 @@
       </c>
       <c r="Y54" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/360-residences-san-jose-ca/xx7h13n/</t>
+        </is>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/san-jose/360-residences</t>
         </is>
       </c>
@@ -16158,7 +16888,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>The Fay (SoFA Luxury Tower)</t>
+          <t>Flow San Jose (formerly The Fay)</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -16255,7 +16985,12 @@
       </c>
       <c r="Y55" s="3" t="inlineStr">
         <is>
-          <t>https://www.thefaysj.com/</t>
+          <t>https://www.apartments.com/flow-san-jose-san-jose-ca/12knvq5/</t>
+        </is>
+      </c>
+      <c r="Z55" s="3" t="inlineStr">
+        <is>
+          <t>https://flow.life/en/properties/san-jose</t>
         </is>
       </c>
     </row>
@@ -16359,12 +17094,17 @@
       </c>
       <c r="X56" s="3" t="inlineStr">
         <is>
-          <t>715 W Julian St, San Jose, CA 95126</t>
+          <t>717 W Julian St, San Jose, CA 95126</t>
         </is>
       </c>
       <c r="Y56" s="3" t="inlineStr">
         <is>
-          <t>https://www.diridonwest.com/</t>
+          <t>https://www.apartments.com/diridon-west-san-jose-ca/l194cvd/</t>
+        </is>
+      </c>
+      <c r="Z56" s="3" t="inlineStr">
+        <is>
+          <t>https://diridonwest.com/</t>
         </is>
       </c>
     </row>
@@ -16376,7 +17116,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Modera The Alameda</t>
+          <t>787 The Alameda (formerly Modera The Alameda)</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -16473,7 +17213,12 @@
       </c>
       <c r="Y57" s="3" t="inlineStr">
         <is>
-          <t>https://www.millcreekplaces.com/community/modera-the-alameda/</t>
+          <t>https://www.apartments.com/787-the-alameda-san-jose-ca/7f64s5w/</t>
+        </is>
+      </c>
+      <c r="Z57" s="3" t="inlineStr">
+        <is>
+          <t>https://www.787thealameda.com/</t>
         </is>
       </c>
     </row>
@@ -16485,7 +17230,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Avalon Morrison Park</t>
+          <t>Bell Diridon (formerly Avalon Morrison Park)</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -16584,7 +17329,12 @@
       </c>
       <c r="Y58" s="3" t="inlineStr">
         <is>
-          <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-morrison-park/</t>
+          <t>https://www.apartments.com/bell-diridon-san-jose-ca/q9197cx/</t>
+        </is>
+      </c>
+      <c r="Z58" s="3" t="inlineStr">
+        <is>
+          <t>https://www.belldiridon.com/</t>
         </is>
       </c>
     </row>
@@ -16693,7 +17443,12 @@
       </c>
       <c r="Y59" s="2" t="inlineStr">
         <is>
-          <t>https://www.meridianmidtown.com/</t>
+          <t>https://www.apartments.com/meridian-at-midtown-san-jose-ca/ezyhf1m/</t>
+        </is>
+      </c>
+      <c r="Z59" s="2" t="inlineStr">
+        <is>
+          <t>https://meridianmidtown.com/</t>
         </is>
       </c>
     </row>
@@ -16804,6 +17559,11 @@
       </c>
       <c r="Y60" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/embark-apartments-fremont-ca/c2hfn5g/</t>
+        </is>
+      </c>
+      <c r="Z60" s="3" t="inlineStr">
+        <is>
           <t>https://www.embarkapartments.com/</t>
         </is>
       </c>
@@ -16816,7 +17576,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Amara at Tasman East</t>
+          <t>Marina Playa Apartment Homes</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -16893,7 +17653,7 @@
       </c>
       <c r="U61" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Active Community (Greystar))</t>
+          <t>UDR (Verified Active Community (Greystar))</t>
         </is>
       </c>
       <c r="V61" s="3" t="inlineStr">
@@ -16908,12 +17668,17 @@
       </c>
       <c r="X61" s="3" t="inlineStr">
         <is>
-          <t>2233 Calle Del Mundo, Santa Clara, CA 95054</t>
+          <t>3500 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y61" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com/</t>
+          <t>https://www.apartments.com/marina-playa-santa-clara-ca/d6tg4dk/</t>
+        </is>
+      </c>
+      <c r="Z61" s="3" t="inlineStr">
+        <is>
+          <t>https://www.udr.com/san-francisco-bay-area-apartments/santa-clara/marina-playa/</t>
         </is>
       </c>
     </row>
@@ -17019,12 +17784,17 @@
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t>2250 Monroe St, Santa Clara, CA 95050</t>
+          <t>4500 Carlyle Ct, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y62" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/the-carlyle-santa-clara-ca/</t>
+          <t>https://www.apartments.com/carlyle-santa-clara-ca/j7b5mj7/</t>
+        </is>
+      </c>
+      <c r="Z62" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thecarlyle-apartments.com/</t>
         </is>
       </c>
     </row>
@@ -17042,7 +17812,7 @@
     <col min="17" max="20" width="13" customWidth="1"/>
     <col min="21" max="21" width="28" customWidth="1"/>
     <col min="22" max="23" width="46" customWidth="1"/>
-    <col min="24" max="25" width="36" customWidth="1"/>
+    <col min="24" max="26" width="38" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -17168,6 +17938,11 @@
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
+          <t>Apartments.com Listing</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
           <t>Official Website</t>
         </is>
       </c>
@@ -17277,7 +18052,12 @@
       </c>
       <c r="Y2" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com</t>
+          <t>https://www.apartments.com/passero-santa-clara-ca/vbeyz4d/</t>
+        </is>
+      </c>
+      <c r="Z2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livepassero.com/</t>
         </is>
       </c>
     </row>
@@ -17388,7 +18168,12 @@
       </c>
       <c r="Y3" s="3" t="inlineStr">
         <is>
-          <t>https://www.equityapartments.com/san-francisco-bay-area/santa-clara/estancia-at-santa-clara-apartments</t>
+          <t>https://www.apartments.com/estancia-at-santa-clara-santa-clara-ca/bfd2x09/</t>
+        </is>
+      </c>
+      <c r="Z3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/estancia-at-santa-clara-apartments</t>
         </is>
       </c>
     </row>
@@ -17499,6 +18284,11 @@
       </c>
       <c r="Y4" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/river-terrace-santa-clara-ca/dcr4v1l/</t>
+        </is>
+      </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
           <t>https://www.udr.com/san-francisco-bay-area-apartments/santa-clara/river-terrace/</t>
         </is>
       </c>
@@ -17610,7 +18400,12 @@
       </c>
       <c r="Y5" s="2" t="inlineStr">
         <is>
-          <t>https://www.liveprado.com</t>
+          <t>https://www.apartments.com/prado-santa-clara-ca/b8re69b/</t>
+        </is>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liveprado.com/</t>
         </is>
       </c>
     </row>
@@ -17721,7 +18516,12 @@
       </c>
       <c r="Y6" s="2" t="inlineStr">
         <is>
-          <t>https://www.villasontheboulevard.com</t>
+          <t>https://www.apartments.com/villas-on-the-boulevard-santa-clara-ca/xpzkmpn/</t>
+        </is>
+      </c>
+      <c r="Z6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.villasontheboulevard.com/</t>
         </is>
       </c>
     </row>
@@ -17832,7 +18632,12 @@
       </c>
       <c r="Y7" s="4" t="inlineStr">
         <is>
-          <t>https://www.prometheusapartments.com/santa-clara-ca/mansion-grove/</t>
+          <t>https://www.apartments.com/mansion-grove-santa-clara-ca/l36cb4f/</t>
+        </is>
+      </c>
+      <c r="Z7" s="4" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/mansion-grove/</t>
         </is>
       </c>
     </row>
@@ -17941,6 +18746,11 @@
       </c>
       <c r="Y8" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/santa-clara-square-apartment-homes-santa-clara-ca/rqgtnx3/</t>
+        </is>
+      </c>
+      <c r="Z8" s="3" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/santa-clara/santa-clara-square.html</t>
         </is>
       </c>
@@ -17953,7 +18763,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Riva Terra Apartments</t>
+          <t>Bella Vista Apartments</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -18032,7 +18842,7 @@
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Institutional Community)</t>
+          <t>Interstate Equities / Bella Vista (Verified Institutional Community)</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
@@ -18047,12 +18857,17 @@
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>2900 Lakeside Dr, Santa Clara, CA 95054</t>
+          <t>1500 Vista Club Cir, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y9" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/riva-terra-santa-clara-ca/65k9eeu/</t>
+          <t>https://www.apartments.com/bella-vista-santa-clara-ca/lc3w7ng/</t>
+        </is>
+      </c>
+      <c r="Z9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bellavista-apartments.com/</t>
         </is>
       </c>
     </row>
@@ -18064,7 +18879,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Station 1 (Lawrence Station)</t>
+          <t>Marina Cove Apartment Homes</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -18141,7 +18956,7 @@
       </c>
       <c r="U10" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Transit-Oriented Community)</t>
+          <t>Essex Property Trust (Verified Transit-Oriented Community)</t>
         </is>
       </c>
       <c r="V10" s="3" t="inlineStr">
@@ -18156,12 +18971,17 @@
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>3515 Reed Ave, Santa Clara, CA 95051</t>
+          <t>3480 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y10" s="3" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/santa-clara-ca/</t>
+          <t>https://www.apartments.com/marina-cove-santa-clara-ca/gsl8bkx/</t>
+        </is>
+      </c>
+      <c r="Z10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/santa-clara/marina-cove</t>
         </is>
       </c>
     </row>
@@ -18270,7 +19090,12 @@
       </c>
       <c r="Y11" s="3" t="inlineStr">
         <is>
-          <t>https://www.550moreland.com/</t>
+          <t>https://www.apartments.com/550-moreland-santa-clara-ca/ypyh9ns/</t>
+        </is>
+      </c>
+      <c r="Z11" s="3" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/550-moreland</t>
         </is>
       </c>
     </row>
@@ -18379,7 +19204,12 @@
       </c>
       <c r="Y12" s="3" t="inlineStr">
         <is>
-          <t>https://www.aveliving.com/locations/san-francisco-bay-area/santa-clara/ave-santa-clara</t>
+          <t>https://www.apartments.com/ave-santa-clara-santa-clara-ca/z3k89nx/</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.aveliving.com/locations/south-bay-silicon-valley/santa-clara</t>
         </is>
       </c>
     </row>
@@ -18488,7 +19318,12 @@
       </c>
       <c r="Y13" s="3" t="inlineStr">
         <is>
-          <t>https://www.thelafayettesantaclara.com/</t>
+          <t>https://www.apartments.com/the-lafayette-santa-clara-ca/c3enymd/</t>
+        </is>
+      </c>
+      <c r="Z13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.livethelafayette.com/</t>
         </is>
       </c>
     </row>
@@ -18597,7 +19432,12 @@
       </c>
       <c r="Y14" s="2" t="inlineStr">
         <is>
-          <t>https://www.theclaraapartments.com/</t>
+          <t>https://www.apartments.com/the-clara-santa-clara-ca/6b3v70v/</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>https://theclara.com/</t>
         </is>
       </c>
     </row>
@@ -18708,6 +19548,11 @@
       </c>
       <c r="Y15" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/monticello-apartment-homes-santa-clara-ca/svq6gr4/</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
           <t>https://www.irvinecompanyapartments.com/locations/northern-california/santa-clara/monticello.html</t>
         </is>
       </c>
@@ -18817,6 +19662,11 @@
       </c>
       <c r="Y16" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/mylo-santa-clara-santa-clara-ca/1rn76d4/</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/santa-clara/mylo-santa-clara</t>
         </is>
       </c>
@@ -18926,6 +19776,11 @@
       </c>
       <c r="Y17" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/lorien-santa-clara-ca/ls5tjef/</t>
+        </is>
+      </c>
+      <c r="Z17" s="3" t="inlineStr">
+        <is>
           <t>https://www.equityapartments.com/san-francisco-bay/santa-clara/lorien-apartments</t>
         </is>
       </c>
@@ -19037,7 +19892,12 @@
       </c>
       <c r="Y18" s="2" t="inlineStr">
         <is>
-          <t>https://www.deanzaproperties.com/apartments/ca/santa-clara/catalina-luxury-apartments/</t>
+          <t>https://www.apartments.com/catalina-luxury-apartments-santa-clara-ca/5d8x1hm/</t>
+        </is>
+      </c>
+      <c r="Z18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.deanzaproperties.com/south-bay-area/catalina-luxury-apartments/</t>
         </is>
       </c>
     </row>
@@ -19148,6 +20008,11 @@
       </c>
       <c r="Y19" s="2" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/villa-granada-santa-clara-ca/q89dqzw/</t>
+        </is>
+      </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
           <t>https://www.essexapartmenthomes.com/apartments/santa-clara/villa-granada</t>
         </is>
       </c>
@@ -19257,7 +20122,12 @@
       </c>
       <c r="Y20" s="2" t="inlineStr">
         <is>
-          <t>https://www.prometheusapartments.com/ca/santa-clara-apartments/cobalt</t>
+          <t>https://www.apartments.com/cobalt-santa-clara-ca/pnpkzps/</t>
+        </is>
+      </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>https://prometheusapartments.com/ca/santa-clara-apartments/cobalt</t>
         </is>
       </c>
     </row>
@@ -19366,7 +20236,12 @@
       </c>
       <c r="Y21" s="3" t="inlineStr">
         <is>
-          <t>https://www.hollandresidential.com/ca/santa-clara/orlo</t>
+          <t>https://www.apartments.com/orlo-and-alba-santa-clara-ca/1pw4vv6/</t>
+        </is>
+      </c>
+      <c r="Z21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.hollandresidential.com/ca/santa-clara/orlo-alba</t>
         </is>
       </c>
     </row>
@@ -19475,6 +20350,11 @@
       </c>
       <c r="Y22" s="3" t="inlineStr">
         <is>
+          <t>https://www.apartments.com/domicilio-santa-clara-ca/6x81pwt/</t>
+        </is>
+      </c>
+      <c r="Z22" s="3" t="inlineStr">
+        <is>
           <t>https://www.domicilioapts.com/</t>
         </is>
       </c>
@@ -19487,7 +20367,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Amara at Tasman East</t>
+          <t>Marina Playa Apartment Homes</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -19564,7 +20444,7 @@
       </c>
       <c r="U23" s="3" t="inlineStr">
         <is>
-          <t>Greystar (Verified Active Community (Greystar))</t>
+          <t>UDR (Verified Active Community (Greystar))</t>
         </is>
       </c>
       <c r="V23" s="3" t="inlineStr">
@@ -19579,12 +20459,17 @@
       </c>
       <c r="X23" s="3" t="inlineStr">
         <is>
-          <t>2233 Calle Del Mundo, Santa Clara, CA 95054</t>
+          <t>3500 Granada Ave, Santa Clara, CA 95051</t>
         </is>
       </c>
       <c r="Y23" s="3" t="inlineStr">
         <is>
-          <t>https://www.greystar.com/</t>
+          <t>https://www.apartments.com/marina-playa-santa-clara-ca/d6tg4dk/</t>
+        </is>
+      </c>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.udr.com/san-francisco-bay-area-apartments/santa-clara/marina-playa/</t>
         </is>
       </c>
     </row>
@@ -19690,12 +20575,17 @@
       </c>
       <c r="X24" s="2" t="inlineStr">
         <is>
-          <t>2250 Monroe St, Santa Clara, CA 95050</t>
+          <t>4500 Carlyle Ct, Santa Clara, CA 95054</t>
         </is>
       </c>
       <c r="Y24" s="2" t="inlineStr">
         <is>
-          <t>https://www.apartments.com/the-carlyle-santa-clara-ca/</t>
+          <t>https://www.apartments.com/carlyle-santa-clara-ca/j7b5mj7/</t>
+        </is>
+      </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.thecarlyle-apartments.com/</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add 15 outer-ring verified apartments (131 total)
</commit_message>
<xml_diff>
--- a/San_Jose_Apartments_Tracker.xlsx
+++ b/San_Jose_Apartments_Tracker.xlsx
@@ -13547,6 +13547,1732 @@
         </is>
       </c>
     </row>
+    <row r="118" ht="42" customHeight="1">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Aya Apartments</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
+        <is>
+          <t>Walk to Warm Springs BART + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E118" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="F118" s="3">
+        <v>14</v>
+      </c>
+      <c r="G118" s="3" t="inlineStr">
+        <is>
+          <t>24m total (4m walk → 15m BART Southbound → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H118" s="3">
+        <v>3100</v>
+      </c>
+      <c r="I118" s="3" t="inlineStr">
+        <is>
+          <t>655</t>
+        </is>
+      </c>
+      <c r="J118" s="3">
+        <v>3256</v>
+      </c>
+      <c r="K118" s="3" t="inlineStr">
+        <is>
+          <t>678–775</t>
+        </is>
+      </c>
+      <c r="L118" s="3">
+        <v>0</v>
+      </c>
+      <c r="M118" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N118" s="3">
+        <v>210</v>
+      </c>
+      <c r="O118" s="3">
+        <v>3310</v>
+      </c>
+      <c r="P118" s="3">
+        <v>3466</v>
+      </c>
+      <c r="Q118" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R118" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S118" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T118" s="3">
+        <v>4.1</v>
+      </c>
+      <c r="U118" s="3" t="inlineStr">
+        <is>
+          <t>MG Properties (Verified Market-Rate Luxury Community (2022 Build))</t>
+        </is>
+      </c>
+      <c r="V118" s="3" t="inlineStr">
+        <is>
+          <t>Walk 4 minutes to Warm Springs BART (1 stop to Milpitas BART -&gt; VTA Orange Line to Cisco Way) or hop straight down I-880 S; includes $0 free garage parking and huge 655 sq ft studios.</t>
+        </is>
+      </c>
+      <c r="W118" s="3" t="inlineStr">
+        <is>
+          <t>Limited immediate late-night restaurants on surrounding Warm Springs Innovation District blocks; occasional BART track dust on outward-facing balconies.</t>
+        </is>
+      </c>
+      <c r="X118" s="3" t="inlineStr">
+        <is>
+          <t>45147 Lopes Rd, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/aya-apartments-fremont-ca/wxez1gh/</t>
+        </is>
+      </c>
+      <c r="Z118" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ayaapts.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="42" customHeight="1">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B119" s="3" t="inlineStr">
+        <is>
+          <t>Leya Apartments</t>
+        </is>
+      </c>
+      <c r="C119" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D119" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Brand-New + $2,950 Studio + $0 Park</t>
+        </is>
+      </c>
+      <c r="E119" s="3">
+        <v>8.7</v>
+      </c>
+      <c r="F119" s="3">
+        <v>14</v>
+      </c>
+      <c r="G119" s="3" t="inlineStr">
+        <is>
+          <t>26m total (6m walk → 15m BART Southbound → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H119" s="3">
+        <v>2950</v>
+      </c>
+      <c r="I119" s="3" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="J119" s="3">
+        <v>3130</v>
+      </c>
+      <c r="K119" s="3" t="inlineStr">
+        <is>
+          <t>690–780</t>
+        </is>
+      </c>
+      <c r="L119" s="3">
+        <v>0</v>
+      </c>
+      <c r="M119" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N119" s="3">
+        <v>210</v>
+      </c>
+      <c r="O119" s="3">
+        <v>3160</v>
+      </c>
+      <c r="P119" s="3">
+        <v>3340</v>
+      </c>
+      <c r="Q119" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R119" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S119" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T119" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U119" s="3" t="inlineStr">
+        <is>
+          <t>Quarterra Multifamily (Verified Market-Rate Luxury Community (2023 Build))</t>
+        </is>
+      </c>
+      <c r="V119" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ rating! Brand-new luxury finishes with Studios under $3,000 ($2,950), $0 included garage parking, up to 6 weeks free, and walkable to Warm Springs BART.</t>
+        </is>
+      </c>
+      <c r="W119" s="3" t="inlineStr">
+        <is>
+          <t>Occasional early-morning commercial/construction truck noise along Innovation Way.</t>
+        </is>
+      </c>
+      <c r="X119" s="3" t="inlineStr">
+        <is>
+          <t>3301 Innovation Way, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/leya-fremont-ca/mkzbh5l/</t>
+        </is>
+      </c>
+      <c r="Z119" s="3" t="inlineStr">
+        <is>
+          <t>https://www.liveleya.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="42" customHeight="1">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>eaves Fremont</t>
+        </is>
+      </c>
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay 1BR at $2,850 + $0 Parking</t>
+        </is>
+      </c>
+      <c r="E120" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="F120" s="2">
+        <v>16</v>
+      </c>
+      <c r="G120" s="2" t="inlineStr">
+        <is>
+          <t>31m total (8m walk → 18m Bus 251 / Bike to Warm Springs BART → Milpitas VTA Orange Line → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I120" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J120" s="2">
+        <v>2850</v>
+      </c>
+      <c r="K120" s="2" t="inlineStr">
+        <is>
+          <t>701–901</t>
+        </is>
+      </c>
+      <c r="L120" s="2">
+        <v>0</v>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N120" s="2">
+        <v>205</v>
+      </c>
+      <c r="O120" s="2">
+        <v>3055</v>
+      </c>
+      <c r="P120" s="2">
+        <v>3055</v>
+      </c>
+      <c r="Q120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S120" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T120" s="2">
+        <v>3.6</v>
+      </c>
+      <c r="U120" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities (Verified Market-Rate Garden Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V120" s="2" t="inlineStr">
+        <is>
+          <t>True sub-$2,900 1-Bedroom ($2,850 for 701–901 sq ft) managed by AvalonBay with $0 included parking in quiet, safe Warm Springs / Mission San Jose.</t>
+        </is>
+      </c>
+      <c r="W120" s="2" t="inlineStr">
+        <is>
+          <t>Older 1980s garden-style wood framing; open guest parking fills up in the evening.</t>
+        </is>
+      </c>
+      <c r="X120" s="2" t="inlineStr">
+        <is>
+          <t>231 Woodcreek Cmn, Fremont, CA 94539</t>
+        </is>
+      </c>
+      <c r="Y120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/eaves-fremont-fremont-ca/w4ek4pk/</t>
+        </is>
+      </c>
+      <c r="Z120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.avaloncommunities.com/california/fremont-apartments/eaves-fremont/</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="42" customHeight="1">
+      <c r="A121" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B121" s="3" t="inlineStr">
+        <is>
+          <t>The Tolman</t>
+        </is>
+      </c>
+      <c r="C121" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D121" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Luxury 1BR $2,695 / Studio $2,420 ($0 Park)</t>
+        </is>
+      </c>
+      <c r="E121" s="3">
+        <v>12.7</v>
+      </c>
+      <c r="F121" s="3">
+        <v>19</v>
+      </c>
+      <c r="G121" s="3" t="inlineStr">
+        <is>
+          <t>32m total (6m walk → 21m BART Orange/Green Line → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H121" s="3">
+        <v>2420</v>
+      </c>
+      <c r="I121" s="3" t="inlineStr">
+        <is>
+          <t>549</t>
+        </is>
+      </c>
+      <c r="J121" s="3">
+        <v>2695</v>
+      </c>
+      <c r="K121" s="3" t="inlineStr">
+        <is>
+          <t>688–748</t>
+        </is>
+      </c>
+      <c r="L121" s="3">
+        <v>0</v>
+      </c>
+      <c r="M121" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N121" s="3">
+        <v>205</v>
+      </c>
+      <c r="O121" s="3">
+        <v>2625</v>
+      </c>
+      <c r="P121" s="3">
+        <v>2900</v>
+      </c>
+      <c r="Q121" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R121" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S121" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T121" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U121" s="3" t="inlineStr">
+        <is>
+          <t>Woodmont Real Estate Services (Verified Market-Rate Luxury Community)</t>
+        </is>
+      </c>
+      <c r="V121" s="3" t="inlineStr">
+        <is>
+          <t>Phenomenal luxury value just north of Warm Springs: 4.4★ rating, Studios at $2,420 and 1BRs at $2,695 with $0 free garage parking and direct BART access to Milpitas/VTA!</t>
+        </is>
+      </c>
+      <c r="W121" s="3" t="inlineStr">
+        <is>
+          <t>Slightly longer 13-mile I-880 S drive to Cisco compared to Warm Springs/Milpitas; standard arterial traffic on Fremont Blvd.</t>
+        </is>
+      </c>
+      <c r="X121" s="3" t="inlineStr">
+        <is>
+          <t>39176 Fremont Blvd, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-tolman-fremont-ca/4flaayc/</t>
+        </is>
+      </c>
+      <c r="Z121" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thetolmanapts.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="42" customHeight="1">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>The Martin at CityLine</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D122" s="3" t="inlineStr">
+        <is>
+          <t>4.3★ Brand-New Downtown Sunnyvale CityLine</t>
+        </is>
+      </c>
+      <c r="E122" s="3">
+        <v>8.4</v>
+      </c>
+      <c r="F122" s="3">
+        <v>14</v>
+      </c>
+      <c r="G122" s="3" t="inlineStr">
+        <is>
+          <t>29m total (3m walk → 21m VTA Bus 55 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H122" s="3">
+        <v>3325</v>
+      </c>
+      <c r="I122" s="3" t="inlineStr">
+        <is>
+          <t>524–536</t>
+        </is>
+      </c>
+      <c r="J122" s="3">
+        <v>3495</v>
+      </c>
+      <c r="K122" s="3" t="inlineStr">
+        <is>
+          <t>694–958</t>
+        </is>
+      </c>
+      <c r="L122" s="3">
+        <v>100</v>
+      </c>
+      <c r="M122" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N122" s="3">
+        <v>215</v>
+      </c>
+      <c r="O122" s="3">
+        <v>3640</v>
+      </c>
+      <c r="P122" s="3">
+        <v>3810</v>
+      </c>
+      <c r="Q122" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R122" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S122" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T122" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="U122" s="3" t="inlineStr">
+        <is>
+          <t>Sares-Regis Group (Verified Market-Rate Luxury High-Rise (2024 Build))</t>
+        </is>
+      </c>
+      <c r="V122" s="3" t="inlineStr">
+        <is>
+          <t>4.3★ brand-new 2024 luxury building right in the heart of CityLine Sunnyvale — Whole Foods, Target, AMC Theater, and 30+ Murphy Ave restaurants are literally downstairs!</t>
+        </is>
+      </c>
+      <c r="W122" s="3" t="inlineStr">
+        <is>
+          <t>Unbundled $100/mo garage parking; 1BRs quickly climb above $3,500 (target the 536 sq ft Studios with 4 weeks free).</t>
+        </is>
+      </c>
+      <c r="X122" s="3" t="inlineStr">
+        <is>
+          <t>240 S Taaffe St, Sunnyvale, CA 94086</t>
+        </is>
+      </c>
+      <c r="Y122" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-martin-sunnyvale-ca-94086/enp0vt6/</t>
+        </is>
+      </c>
+      <c r="Z122" s="3" t="inlineStr">
+        <is>
+          <t>https://livethemartin.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="42" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>Arioso Apartments</t>
+        </is>
+      </c>
+      <c r="C123" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>Across from Apple Park + $0 Underground Garage</t>
+        </is>
+      </c>
+      <c r="E123" s="2">
+        <v>9.4</v>
+      </c>
+      <c r="F123" s="2">
+        <v>19</v>
+      </c>
+      <c r="G123" s="2" t="inlineStr">
+        <is>
+          <t>35m total (3m walk → 27m VTA Bus 56 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H123" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I123" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J123" s="2">
+        <v>3359</v>
+      </c>
+      <c r="K123" s="2" t="inlineStr">
+        <is>
+          <t>534–829</t>
+        </is>
+      </c>
+      <c r="L123" s="2">
+        <v>0</v>
+      </c>
+      <c r="M123" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N123" s="2">
+        <v>210</v>
+      </c>
+      <c r="O123" s="2">
+        <v>3569</v>
+      </c>
+      <c r="P123" s="2">
+        <v>3569</v>
+      </c>
+      <c r="Q123" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R123" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S123" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T123" s="2">
+        <v>3.8</v>
+      </c>
+      <c r="U123" s="2" t="inlineStr">
+        <is>
+          <t>Willow Bridge Property Company (Verified Market-Rate Luxury Community)</t>
+        </is>
+      </c>
+      <c r="V123" s="2" t="inlineStr">
+        <is>
+          <t>Prime Cupertino address directly across from Apple Park and walkable to Main Street Cupertino dining, with $0 included underground garage parking.</t>
+        </is>
+      </c>
+      <c r="W123" s="2" t="inlineStr">
+        <is>
+          <t>Limited visitor parking spaces; annual lease renewal increases.</t>
+        </is>
+      </c>
+      <c r="X123" s="2" t="inlineStr">
+        <is>
+          <t>19608 Pruneridge Ave, Cupertino, CA 95014</t>
+        </is>
+      </c>
+      <c r="Y123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/arioso-cupertino-ca/dxEaLh0/</t>
+        </is>
+      </c>
+      <c r="Z123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ariosoapartments.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="42" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>City Gate at Cupertino</t>
+        </is>
+      </c>
+      <c r="C124" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>Walk to Main St Cupertino + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E124" s="2">
+        <v>9.9</v>
+      </c>
+      <c r="F124" s="2">
+        <v>19</v>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>36m total (3m walk → 28m VTA Bus 56 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J124" s="2">
+        <v>3241</v>
+      </c>
+      <c r="K124" s="2" t="inlineStr">
+        <is>
+          <t>728–774</t>
+        </is>
+      </c>
+      <c r="L124" s="2">
+        <v>0</v>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N124" s="2">
+        <v>210</v>
+      </c>
+      <c r="O124" s="2">
+        <v>3451</v>
+      </c>
+      <c r="P124" s="2">
+        <v>3451</v>
+      </c>
+      <c r="Q124" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R124" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S124" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T124" s="2">
+        <v>3.5</v>
+      </c>
+      <c r="U124" s="2" t="inlineStr">
+        <is>
+          <t>Equity Residential (Verified Market-Rate Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V124" s="2" t="inlineStr">
+        <is>
+          <t>Steps from Main Street Cupertino restaurants, Philz Coffee, and Target; spacious 728–774 sq ft 1BRs with $0 included underground parking.</t>
+        </is>
+      </c>
+      <c r="W124" s="2" t="inlineStr">
+        <is>
+          <t>Stevens Creek Blvd traffic noise on south-facing balconies (choose a courtyard-facing unit).</t>
+        </is>
+      </c>
+      <c r="X124" s="2" t="inlineStr">
+        <is>
+          <t>5608 Stevens Creek Blvd, Cupertino, CA 95014</t>
+        </is>
+      </c>
+      <c r="Y124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/city-gate-at-cupertino-cupertino-ca/l17q0p2/</t>
+        </is>
+      </c>
+      <c r="Z124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.equityapartments.com/san-francisco-bay-area/cupertino/city-gate-at-cupertino-apartments</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="42" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>The Villages at Cupertino</t>
+        </is>
+      </c>
+      <c r="C125" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>27-Acre Cupertino Park Setting + $0 Park</t>
+        </is>
+      </c>
+      <c r="E125" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="F125" s="2">
+        <v>22</v>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>37m total (5m walk → 27m VTA Bus 55 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H125" s="2">
+        <v>3212</v>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
+        <is>
+          <t>506</t>
+        </is>
+      </c>
+      <c r="J125" s="2">
+        <v>3495</v>
+      </c>
+      <c r="K125" s="2" t="inlineStr">
+        <is>
+          <t>680–730</t>
+        </is>
+      </c>
+      <c r="L125" s="2">
+        <v>0</v>
+      </c>
+      <c r="M125" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N125" s="2">
+        <v>205</v>
+      </c>
+      <c r="O125" s="2">
+        <v>3417</v>
+      </c>
+      <c r="P125" s="2">
+        <v>3700</v>
+      </c>
+      <c r="Q125" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R125" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S125" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T125" s="2">
+        <v>3.9</v>
+      </c>
+      <c r="U125" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Real Estate Group (Verified Market-Rate Garden Community)</t>
+        </is>
+      </c>
+      <c r="V125" s="2" t="inlineStr">
+        <is>
+          <t>Massive 27-acre green park setting in Cupertino with tennis courts, Prometheus management, $0 included parking, and up to 3 weeks free.</t>
+        </is>
+      </c>
+      <c r="W125" s="2" t="inlineStr">
+        <is>
+          <t>Older vintage wood-frame construction (request an upper-floor unit to avoid upstairs footsteps).</t>
+        </is>
+      </c>
+      <c r="X125" s="2" t="inlineStr">
+        <is>
+          <t>20875 Valley Green Dr, Cupertino, CA 95014</t>
+        </is>
+      </c>
+      <c r="Y125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/villages-at-cupertino-cupertino-ca/xc_7t2j/</t>
+        </is>
+      </c>
+      <c r="Z125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.prometheusapartments.com/ca/cupertino-apartments/villages-at-cupertino/</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="42" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Americana Apartments</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>Direct Hwy 237 East Shot + VTA Orange Line</t>
+        </is>
+      </c>
+      <c r="E126" s="2">
+        <v>9.1</v>
+      </c>
+      <c r="F126" s="2">
+        <v>14</v>
+      </c>
+      <c r="G126" s="2" t="inlineStr">
+        <is>
+          <t>33m total (7m walk → 21m VTA Orange Line → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I126" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J126" s="2">
+        <v>3243</v>
+      </c>
+      <c r="K126" s="2" t="inlineStr">
+        <is>
+          <t>610–750</t>
+        </is>
+      </c>
+      <c r="L126" s="2">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N126" s="2">
+        <v>210</v>
+      </c>
+      <c r="O126" s="2">
+        <v>3453</v>
+      </c>
+      <c r="P126" s="2">
+        <v>3453</v>
+      </c>
+      <c r="Q126" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R126" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S126" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T126" s="2">
+        <v>3.8</v>
+      </c>
+      <c r="U126" s="2" t="inlineStr">
+        <is>
+          <t>Prometheus Real Estate Group (Verified Market-Rate Garden Community)</t>
+        </is>
+      </c>
+      <c r="V126" s="2" t="inlineStr">
+        <is>
+          <t>Sits right at the Hwy 237 / Hwy 85 junction for a straight shot east on Hwy 237 to Cisco Way, plus direct VTA Orange Line access and $0 parking.</t>
+        </is>
+      </c>
+      <c r="W126" s="2" t="inlineStr">
+        <is>
+          <t>Carport parking rather than fully enclosed underground garage; standard Prometheus move-out cleaning deductions.</t>
+        </is>
+      </c>
+      <c r="X126" s="2" t="inlineStr">
+        <is>
+          <t>707 Continental Cir, Mountain View, CA 94040</t>
+        </is>
+      </c>
+      <c r="Y126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/americana-apartments-mountain-view-ca/peO12Fv/</t>
+        </is>
+      </c>
+      <c r="Z126" s="2" t="inlineStr">
+        <is>
+          <t>https://liveatamericana.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="42" customHeight="1">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B127" s="3" t="inlineStr">
+        <is>
+          <t>300 Railway</t>
+        </is>
+      </c>
+      <c r="C127" s="3" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D127" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Walkable Downtown Campbell + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E127" s="3">
+        <v>11.8</v>
+      </c>
+      <c r="F127" s="3">
+        <v>17</v>
+      </c>
+      <c r="G127" s="3" t="inlineStr">
+        <is>
+          <t>36m total (2m walk → 29m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H127" s="3">
+        <v>2975</v>
+      </c>
+      <c r="I127" s="3" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
+      </c>
+      <c r="J127" s="3">
+        <v>3450</v>
+      </c>
+      <c r="K127" s="3" t="inlineStr">
+        <is>
+          <t>680–745</t>
+        </is>
+      </c>
+      <c r="L127" s="3">
+        <v>0</v>
+      </c>
+      <c r="M127" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N127" s="3">
+        <v>205</v>
+      </c>
+      <c r="O127" s="3">
+        <v>3180</v>
+      </c>
+      <c r="P127" s="3">
+        <v>3655</v>
+      </c>
+      <c r="Q127" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R127" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S127" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T127" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U127" s="3" t="inlineStr">
+        <is>
+          <t>St. Anton Multifamily (Verified Market-Rate Community)</t>
+        </is>
+      </c>
+      <c r="V127" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ rating right in walkable Downtown Campbell! Step out your door to Campbell Ave cafes, Los Gatos Creek Trail, and Downtown Campbell VTA Light Rail, with $0 free garage parking.</t>
+        </is>
+      </c>
+      <c r="W127" s="3" t="inlineStr">
+        <is>
+          <t>Studios are cozy (441 sq ft); light rail bell audible when windows are open.</t>
+        </is>
+      </c>
+      <c r="X127" s="3" t="inlineStr">
+        <is>
+          <t>300 Railway Ave, Campbell, CA 95008</t>
+        </is>
+      </c>
+      <c r="Y127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/300-railway-campbell-ca/bj6kr9b/</t>
+        </is>
+      </c>
+      <c r="Z127" s="3" t="inlineStr">
+        <is>
+          <t>https://www.300railway.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="42" customHeight="1">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>The Parc at Pruneyard</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>Across from Campbell Pruneyard Trader Joe's</t>
+        </is>
+      </c>
+      <c r="E128" s="2">
+        <v>12.4</v>
+      </c>
+      <c r="F128" s="2">
+        <v>20</v>
+      </c>
+      <c r="G128" s="2" t="inlineStr">
+        <is>
+          <t>40m total (6m walk → 29m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I128" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J128" s="2">
+        <v>3397</v>
+      </c>
+      <c r="K128" s="2" t="inlineStr">
+        <is>
+          <t>750</t>
+        </is>
+      </c>
+      <c r="L128" s="2">
+        <v>0</v>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N128" s="2">
+        <v>210</v>
+      </c>
+      <c r="O128" s="2">
+        <v>3607</v>
+      </c>
+      <c r="P128" s="2">
+        <v>3607</v>
+      </c>
+      <c r="Q128" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R128" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S128" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T128" s="2">
+        <v>3.7</v>
+      </c>
+      <c r="U128" s="2" t="inlineStr">
+        <is>
+          <t>Essex Property Trust (Verified Market-Rate Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V128" s="2" t="inlineStr">
+        <is>
+          <t>Walk across the street to The Pruneyard (Trader Joe's, Mendocino Farms, Rock Bottom, CineArts) and Los Gatos Creek Trail; $0 included parking.</t>
+        </is>
+      </c>
+      <c r="W128" s="2" t="inlineStr">
+        <is>
+          <t>Older wood-frame floors can transmit upstairs footsteps; tight evening guest parking.</t>
+        </is>
+      </c>
+      <c r="X128" s="2" t="inlineStr">
+        <is>
+          <t>225 Union Ave, Campbell, CA 95008</t>
+        </is>
+      </c>
+      <c r="Y128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-parc-at-pruneyard-campbell-ca/h07w213/</t>
+        </is>
+      </c>
+      <c r="Z128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.essexapartmenthomes.com/apartments/campbell/the-parc-at-pruneyard</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="42" customHeight="1">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>The Franciscan Apartments</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>4.0★ Renovated Campbell 1BR ($3,072 + $0 Park)</t>
+        </is>
+      </c>
+      <c r="E129" s="2">
+        <v>12.5</v>
+      </c>
+      <c r="F129" s="2">
+        <v>19</v>
+      </c>
+      <c r="G129" s="2" t="inlineStr">
+        <is>
+          <t>41m total (9m walk → 27m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H129" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I129" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J129" s="2">
+        <v>3072</v>
+      </c>
+      <c r="K129" s="2" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
+      <c r="L129" s="2">
+        <v>0</v>
+      </c>
+      <c r="M129" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N129" s="2">
+        <v>205</v>
+      </c>
+      <c r="O129" s="2">
+        <v>3277</v>
+      </c>
+      <c r="P129" s="2">
+        <v>3277</v>
+      </c>
+      <c r="Q129" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R129" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S129" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T129" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="U129" s="2" t="inlineStr">
+        <is>
+          <t>Greystar (Verified Market-Rate Community)</t>
+        </is>
+      </c>
+      <c r="V129" s="2" t="inlineStr">
+        <is>
+          <t>4.0★ Greystar-managed community in Campbell with renovated quartz kitchen islands, $0 included parking, and easy Hwy 17 / I-880 access.</t>
+        </is>
+      </c>
+      <c r="W129" s="2" t="inlineStr">
+        <is>
+          <t>Limited parking for a 2nd vehicle; occasional daytime exterior maintenance noise.</t>
+        </is>
+      </c>
+      <c r="X129" s="2" t="inlineStr">
+        <is>
+          <t>601 Almarida Dr, Campbell, CA 95008</t>
+        </is>
+      </c>
+      <c r="Y129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-franciscan-campbell-ca/w0gt9ql/</t>
+        </is>
+      </c>
+      <c r="Z129" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liveatfranciscan.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="42" customHeight="1">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Maxwell at Bascom</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D130" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ 2024 Build + Up to 8 Weeks Free</t>
+        </is>
+      </c>
+      <c r="E130" s="3">
+        <v>11.5</v>
+      </c>
+      <c r="F130" s="3">
+        <v>17</v>
+      </c>
+      <c r="G130" s="3" t="inlineStr">
+        <is>
+          <t>36m total (4m walk → 27m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H130" s="3">
+        <v>2911</v>
+      </c>
+      <c r="I130" s="3" t="inlineStr">
+        <is>
+          <t>466–587</t>
+        </is>
+      </c>
+      <c r="J130" s="3">
+        <v>3304</v>
+      </c>
+      <c r="K130" s="3" t="inlineStr">
+        <is>
+          <t>607–649</t>
+        </is>
+      </c>
+      <c r="L130" s="3">
+        <v>125</v>
+      </c>
+      <c r="M130" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N130" s="3">
+        <v>215</v>
+      </c>
+      <c r="O130" s="3">
+        <v>3251</v>
+      </c>
+      <c r="P130" s="3">
+        <v>3644</v>
+      </c>
+      <c r="Q130" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R130" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S130" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T130" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="U130" s="3" t="inlineStr">
+        <is>
+          <t>Greystar (Verified Market-Rate Luxury Community (2024 Build))</t>
+        </is>
+      </c>
+      <c r="V130" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ brand-new 2024 luxury construction between Willow Glen and Campbell Pruneyard with Studios under $3,000 ($2,911) and up to 8 weeks free!</t>
+        </is>
+      </c>
+      <c r="W130" s="3" t="inlineStr">
+        <is>
+          <t>Unbundled $125/mo garage parking; request an interior courtyard unit away from S. Bascom Ave.</t>
+        </is>
+      </c>
+      <c r="X130" s="3" t="inlineStr">
+        <is>
+          <t>1350 S Bascom Ave, San Jose, CA 95128</t>
+        </is>
+      </c>
+      <c r="Y130" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/maxwell-at-bascom-san-jose-ca/163qzv7/</t>
+        </is>
+      </c>
+      <c r="Z130" s="3" t="inlineStr">
+        <is>
+          <t>https://maxwellatbascom.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="42" customHeight="1">
+      <c r="A131" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B131" s="3" t="inlineStr">
+        <is>
+          <t>La Terraza Apartments</t>
+        </is>
+      </c>
+      <c r="C131" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D131" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ Huge 825–910 Sq Ft 1BR + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E131" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="F131" s="3">
+        <v>17</v>
+      </c>
+      <c r="G131" s="3" t="inlineStr">
+        <is>
+          <t>35m total (3m walk → 27m VTA Bus 57 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H131" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I131" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J131" s="3">
+        <v>3231</v>
+      </c>
+      <c r="K131" s="3" t="inlineStr">
+        <is>
+          <t>825–910</t>
+        </is>
+      </c>
+      <c r="L131" s="3">
+        <v>0</v>
+      </c>
+      <c r="M131" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N131" s="3">
+        <v>215</v>
+      </c>
+      <c r="O131" s="3">
+        <v>3446</v>
+      </c>
+      <c r="P131" s="3">
+        <v>3446</v>
+      </c>
+      <c r="Q131" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R131" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S131" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T131" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="U131" s="3" t="inlineStr">
+        <is>
+          <t>Greystar (Verified Market-Rate Luxury Community)</t>
+        </is>
+      </c>
+      <c r="V131" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ resident rating! Huge 825–910 sq ft 1BR floor plans with $0 included garage parking, 4–6 weeks free, and instant I-280 access near Santana Row &amp; Mitsuwa.</t>
+        </is>
+      </c>
+      <c r="W131" s="3" t="inlineStr">
+        <is>
+          <t>Weekend guest parking fills up quickly; Saratoga Ave rush-hour traffic near I-280.</t>
+        </is>
+      </c>
+      <c r="X131" s="3" t="inlineStr">
+        <is>
+          <t>470 Saratoga Ave, San Jose, CA 95129</t>
+        </is>
+      </c>
+      <c r="Y131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/la-terraza-san-jose-ca/wucpje8/</t>
+        </is>
+      </c>
+      <c r="Z131" s="3" t="inlineStr">
+        <is>
+          <t>https://www.liveatlaterraza.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="42" customHeight="1">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Avalon Willow Glen</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>4.2★ AvalonBay 1BR at $2,770 + Direct VTA Blue Line</t>
+        </is>
+      </c>
+      <c r="E132" s="3">
+        <v>11.3</v>
+      </c>
+      <c r="F132" s="3">
+        <v>18</v>
+      </c>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>37m total (5m walk → 27m VTA Blue Line → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H132" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I132" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J132" s="3">
+        <v>2770</v>
+      </c>
+      <c r="K132" s="3" t="inlineStr">
+        <is>
+          <t>726–814</t>
+        </is>
+      </c>
+      <c r="L132" s="3">
+        <v>0</v>
+      </c>
+      <c r="M132" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N132" s="3">
+        <v>205</v>
+      </c>
+      <c r="O132" s="3">
+        <v>2975</v>
+      </c>
+      <c r="P132" s="3">
+        <v>2975</v>
+      </c>
+      <c r="Q132" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R132" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S132" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T132" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="U132" s="3" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities (Verified Market-Rate Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V132" s="3" t="inlineStr">
+        <is>
+          <t>4.2★ AvalonBay community where a spacious 726–814 sq ft 1BR starts at just $2,770/mo with $0 free parking AND walks directly to the VTA Blue Line (no transfers to Cisco Way!).</t>
+        </is>
+      </c>
+      <c r="W132" s="3" t="inlineStr">
+        <is>
+          <t>Garden walk-up buildings do not have elevators; unassigned surface spots fill up late at night.</t>
+        </is>
+      </c>
+      <c r="X132" s="3" t="inlineStr">
+        <is>
+          <t>3200 Rubino Dr, San Jose, CA 95125</t>
+        </is>
+      </c>
+      <c r="Y132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/avalon-willow-glen-san-jose-ca/4zfygh5/</t>
+        </is>
+      </c>
+      <c r="Z132" s="3" t="inlineStr">
+        <is>
+          <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-willow-glen/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
@@ -22161,6 +23887,1038 @@
       <c r="Z75" s="3" t="inlineStr">
         <is>
           <t>https://www.liveatnaya.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="42" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Aya Apartments</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Walk to Warm Springs BART + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E76" s="3">
+        <v>8.0</v>
+      </c>
+      <c r="F76" s="3">
+        <v>14</v>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>24m total (4m walk → 15m BART Southbound → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H76" s="3">
+        <v>3100</v>
+      </c>
+      <c r="I76" s="3" t="inlineStr">
+        <is>
+          <t>655</t>
+        </is>
+      </c>
+      <c r="J76" s="3">
+        <v>3256</v>
+      </c>
+      <c r="K76" s="3" t="inlineStr">
+        <is>
+          <t>678–775</t>
+        </is>
+      </c>
+      <c r="L76" s="3">
+        <v>0</v>
+      </c>
+      <c r="M76" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N76" s="3">
+        <v>210</v>
+      </c>
+      <c r="O76" s="3">
+        <v>3310</v>
+      </c>
+      <c r="P76" s="3">
+        <v>3466</v>
+      </c>
+      <c r="Q76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S76" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T76" s="3">
+        <v>4.1</v>
+      </c>
+      <c r="U76" s="3" t="inlineStr">
+        <is>
+          <t>MG Properties (Verified Market-Rate Luxury Community (2022 Build))</t>
+        </is>
+      </c>
+      <c r="V76" s="3" t="inlineStr">
+        <is>
+          <t>Walk 4 minutes to Warm Springs BART (1 stop to Milpitas BART -&gt; VTA Orange Line to Cisco Way) or hop straight down I-880 S; includes $0 free garage parking and huge 655 sq ft studios.</t>
+        </is>
+      </c>
+      <c r="W76" s="3" t="inlineStr">
+        <is>
+          <t>Limited immediate late-night restaurants on surrounding Warm Springs Innovation District blocks; occasional BART track dust on outward-facing balconies.</t>
+        </is>
+      </c>
+      <c r="X76" s="3" t="inlineStr">
+        <is>
+          <t>45147 Lopes Rd, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/aya-apartments-fremont-ca/wxez1gh/</t>
+        </is>
+      </c>
+      <c r="Z76" s="3" t="inlineStr">
+        <is>
+          <t>https://www.ayaapts.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="42" customHeight="1">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="inlineStr">
+        <is>
+          <t>Leya Apartments</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Brand-New + $2,950 Studio + $0 Park</t>
+        </is>
+      </c>
+      <c r="E77" s="3">
+        <v>8.7</v>
+      </c>
+      <c r="F77" s="3">
+        <v>14</v>
+      </c>
+      <c r="G77" s="3" t="inlineStr">
+        <is>
+          <t>26m total (6m walk → 15m BART Southbound → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H77" s="3">
+        <v>2950</v>
+      </c>
+      <c r="I77" s="3" t="inlineStr">
+        <is>
+          <t>576</t>
+        </is>
+      </c>
+      <c r="J77" s="3">
+        <v>3130</v>
+      </c>
+      <c r="K77" s="3" t="inlineStr">
+        <is>
+          <t>690–780</t>
+        </is>
+      </c>
+      <c r="L77" s="3">
+        <v>0</v>
+      </c>
+      <c r="M77" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N77" s="3">
+        <v>210</v>
+      </c>
+      <c r="O77" s="3">
+        <v>3160</v>
+      </c>
+      <c r="P77" s="3">
+        <v>3340</v>
+      </c>
+      <c r="Q77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S77" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T77" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U77" s="3" t="inlineStr">
+        <is>
+          <t>Quarterra Multifamily (Verified Market-Rate Luxury Community (2023 Build))</t>
+        </is>
+      </c>
+      <c r="V77" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ rating! Brand-new luxury finishes with Studios under $3,000 ($2,950), $0 included garage parking, up to 6 weeks free, and walkable to Warm Springs BART.</t>
+        </is>
+      </c>
+      <c r="W77" s="3" t="inlineStr">
+        <is>
+          <t>Occasional early-morning commercial/construction truck noise along Innovation Way.</t>
+        </is>
+      </c>
+      <c r="X77" s="3" t="inlineStr">
+        <is>
+          <t>3301 Innovation Way, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/leya-fremont-ca/mkzbh5l/</t>
+        </is>
+      </c>
+      <c r="Z77" s="3" t="inlineStr">
+        <is>
+          <t>https://www.liveleya.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="42" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Strong Contender</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>eaves Fremont</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay 1BR at $2,850 + $0 Parking</t>
+        </is>
+      </c>
+      <c r="E78" s="2">
+        <v>9.6</v>
+      </c>
+      <c r="F78" s="2">
+        <v>16</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>31m total (8m walk → 18m Bus 251 / Bike to Warm Springs BART → Milpitas VTA Orange Line → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J78" s="2">
+        <v>2850</v>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>701–901</t>
+        </is>
+      </c>
+      <c r="L78" s="2">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N78" s="2">
+        <v>205</v>
+      </c>
+      <c r="O78" s="2">
+        <v>3055</v>
+      </c>
+      <c r="P78" s="2">
+        <v>3055</v>
+      </c>
+      <c r="Q78" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S78" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T78" s="2">
+        <v>3.6</v>
+      </c>
+      <c r="U78" s="2" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities (Verified Market-Rate Garden Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V78" s="2" t="inlineStr">
+        <is>
+          <t>True sub-$2,900 1-Bedroom ($2,850 for 701–901 sq ft) managed by AvalonBay with $0 included parking in quiet, safe Warm Springs / Mission San Jose.</t>
+        </is>
+      </c>
+      <c r="W78" s="2" t="inlineStr">
+        <is>
+          <t>Older 1980s garden-style wood framing; open guest parking fills up in the evening.</t>
+        </is>
+      </c>
+      <c r="X78" s="2" t="inlineStr">
+        <is>
+          <t>231 Woodcreek Cmn, Fremont, CA 94539</t>
+        </is>
+      </c>
+      <c r="Y78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/eaves-fremont-fremont-ca/w4ek4pk/</t>
+        </is>
+      </c>
+      <c r="Z78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.avaloncommunities.com/california/fremont-apartments/eaves-fremont/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="42" customHeight="1">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>The Tolman</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>Milpitas Corridor</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Luxury 1BR $2,695 / Studio $2,420 ($0 Park)</t>
+        </is>
+      </c>
+      <c r="E79" s="3">
+        <v>12.7</v>
+      </c>
+      <c r="F79" s="3">
+        <v>19</v>
+      </c>
+      <c r="G79" s="3" t="inlineStr">
+        <is>
+          <t>32m total (6m walk → 21m BART Orange/Green Line → Milpitas VTA Orange Line to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H79" s="3">
+        <v>2420</v>
+      </c>
+      <c r="I79" s="3" t="inlineStr">
+        <is>
+          <t>549</t>
+        </is>
+      </c>
+      <c r="J79" s="3">
+        <v>2695</v>
+      </c>
+      <c r="K79" s="3" t="inlineStr">
+        <is>
+          <t>688–748</t>
+        </is>
+      </c>
+      <c r="L79" s="3">
+        <v>0</v>
+      </c>
+      <c r="M79" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N79" s="3">
+        <v>205</v>
+      </c>
+      <c r="O79" s="3">
+        <v>2625</v>
+      </c>
+      <c r="P79" s="3">
+        <v>2900</v>
+      </c>
+      <c r="Q79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S79" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T79" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U79" s="3" t="inlineStr">
+        <is>
+          <t>Woodmont Real Estate Services (Verified Market-Rate Luxury Community)</t>
+        </is>
+      </c>
+      <c r="V79" s="3" t="inlineStr">
+        <is>
+          <t>Phenomenal luxury value just north of Warm Springs: 4.4★ rating, Studios at $2,420 and 1BRs at $2,695 with $0 free garage parking and direct BART access to Milpitas/VTA!</t>
+        </is>
+      </c>
+      <c r="W79" s="3" t="inlineStr">
+        <is>
+          <t>Slightly longer 13-mile I-880 S drive to Cisco compared to Warm Springs/Milpitas; standard arterial traffic on Fremont Blvd.</t>
+        </is>
+      </c>
+      <c r="X79" s="3" t="inlineStr">
+        <is>
+          <t>39176 Fremont Blvd, Fremont, CA 94538</t>
+        </is>
+      </c>
+      <c r="Y79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-tolman-fremont-ca/4flaayc/</t>
+        </is>
+      </c>
+      <c r="Z79" s="3" t="inlineStr">
+        <is>
+          <t>https://www.thetolmanapts.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="42" customHeight="1">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>The Martin at CityLine</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>4.3★ Brand-New Downtown Sunnyvale CityLine</t>
+        </is>
+      </c>
+      <c r="E80" s="3">
+        <v>8.4</v>
+      </c>
+      <c r="F80" s="3">
+        <v>14</v>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>29m total (3m walk → 21m VTA Bus 55 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H80" s="3">
+        <v>3325</v>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>524–536</t>
+        </is>
+      </c>
+      <c r="J80" s="3">
+        <v>3495</v>
+      </c>
+      <c r="K80" s="3" t="inlineStr">
+        <is>
+          <t>694–958</t>
+        </is>
+      </c>
+      <c r="L80" s="3">
+        <v>100</v>
+      </c>
+      <c r="M80" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N80" s="3">
+        <v>215</v>
+      </c>
+      <c r="O80" s="3">
+        <v>3640</v>
+      </c>
+      <c r="P80" s="3">
+        <v>3810</v>
+      </c>
+      <c r="Q80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S80" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T80" s="3">
+        <v>4.3</v>
+      </c>
+      <c r="U80" s="3" t="inlineStr">
+        <is>
+          <t>Sares-Regis Group (Verified Market-Rate Luxury High-Rise (2024 Build))</t>
+        </is>
+      </c>
+      <c r="V80" s="3" t="inlineStr">
+        <is>
+          <t>4.3★ brand-new 2024 luxury building right in the heart of CityLine Sunnyvale — Whole Foods, Target, AMC Theater, and 30+ Murphy Ave restaurants are literally downstairs!</t>
+        </is>
+      </c>
+      <c r="W80" s="3" t="inlineStr">
+        <is>
+          <t>Unbundled $100/mo garage parking; 1BRs quickly climb above $3,500 (target the 536 sq ft Studios with 4 weeks free).</t>
+        </is>
+      </c>
+      <c r="X80" s="3" t="inlineStr">
+        <is>
+          <t>240 S Taaffe St, Sunnyvale, CA 94086</t>
+        </is>
+      </c>
+      <c r="Y80" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/the-martin-sunnyvale-ca-94086/enp0vt6/</t>
+        </is>
+      </c>
+      <c r="Z80" s="3" t="inlineStr">
+        <is>
+          <t>https://livethemartin.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="42" customHeight="1">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="inlineStr">
+        <is>
+          <t>300 Railway</t>
+        </is>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>Sunnyvale &amp; Campbell</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ Walkable Downtown Campbell + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E81" s="3">
+        <v>11.8</v>
+      </c>
+      <c r="F81" s="3">
+        <v>17</v>
+      </c>
+      <c r="G81" s="3" t="inlineStr">
+        <is>
+          <t>36m total (2m walk → 29m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H81" s="3">
+        <v>2975</v>
+      </c>
+      <c r="I81" s="3" t="inlineStr">
+        <is>
+          <t>441</t>
+        </is>
+      </c>
+      <c r="J81" s="3">
+        <v>3450</v>
+      </c>
+      <c r="K81" s="3" t="inlineStr">
+        <is>
+          <t>680–745</t>
+        </is>
+      </c>
+      <c r="L81" s="3">
+        <v>0</v>
+      </c>
+      <c r="M81" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N81" s="3">
+        <v>205</v>
+      </c>
+      <c r="O81" s="3">
+        <v>3180</v>
+      </c>
+      <c r="P81" s="3">
+        <v>3655</v>
+      </c>
+      <c r="Q81" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R81" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S81" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T81" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="U81" s="3" t="inlineStr">
+        <is>
+          <t>St. Anton Multifamily (Verified Market-Rate Community)</t>
+        </is>
+      </c>
+      <c r="V81" s="3" t="inlineStr">
+        <is>
+          <t>4.4★ rating right in walkable Downtown Campbell! Step out your door to Campbell Ave cafes, Los Gatos Creek Trail, and Downtown Campbell VTA Light Rail, with $0 free garage parking.</t>
+        </is>
+      </c>
+      <c r="W81" s="3" t="inlineStr">
+        <is>
+          <t>Studios are cozy (441 sq ft); light rail bell audible when windows are open.</t>
+        </is>
+      </c>
+      <c r="X81" s="3" t="inlineStr">
+        <is>
+          <t>300 Railway Ave, Campbell, CA 95008</t>
+        </is>
+      </c>
+      <c r="Y81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/300-railway-campbell-ca/bj6kr9b/</t>
+        </is>
+      </c>
+      <c r="Z81" s="3" t="inlineStr">
+        <is>
+          <t>https://www.300railway.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="42" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Maxwell at Bascom</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ 2024 Build + Up to 8 Weeks Free</t>
+        </is>
+      </c>
+      <c r="E82" s="3">
+        <v>11.5</v>
+      </c>
+      <c r="F82" s="3">
+        <v>17</v>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>36m total (4m walk → 27m VTA Green Line → VTA Blue Line North to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H82" s="3">
+        <v>2911</v>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>466–587</t>
+        </is>
+      </c>
+      <c r="J82" s="3">
+        <v>3304</v>
+      </c>
+      <c r="K82" s="3" t="inlineStr">
+        <is>
+          <t>607–649</t>
+        </is>
+      </c>
+      <c r="L82" s="3">
+        <v>125</v>
+      </c>
+      <c r="M82" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N82" s="3">
+        <v>215</v>
+      </c>
+      <c r="O82" s="3">
+        <v>3251</v>
+      </c>
+      <c r="P82" s="3">
+        <v>3644</v>
+      </c>
+      <c r="Q82" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R82" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S82" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T82" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="U82" s="3" t="inlineStr">
+        <is>
+          <t>Greystar (Verified Market-Rate Luxury Community (2024 Build))</t>
+        </is>
+      </c>
+      <c r="V82" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ brand-new 2024 luxury construction between Willow Glen and Campbell Pruneyard with Studios under $3,000 ($2,911) and up to 8 weeks free!</t>
+        </is>
+      </c>
+      <c r="W82" s="3" t="inlineStr">
+        <is>
+          <t>Unbundled $125/mo garage parking; request an interior courtyard unit away from S. Bascom Ave.</t>
+        </is>
+      </c>
+      <c r="X82" s="3" t="inlineStr">
+        <is>
+          <t>1350 S Bascom Ave, San Jose, CA 95128</t>
+        </is>
+      </c>
+      <c r="Y82" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/maxwell-at-bascom-san-jose-ca/163qzv7/</t>
+        </is>
+      </c>
+      <c r="Z82" s="3" t="inlineStr">
+        <is>
+          <t>https://maxwellatbascom.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="42" customHeight="1">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="inlineStr">
+        <is>
+          <t>La Terraza Apartments</t>
+        </is>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ Huge 825–910 Sq Ft 1BR + $0 Garage</t>
+        </is>
+      </c>
+      <c r="E83" s="3">
+        <v>8.1</v>
+      </c>
+      <c r="F83" s="3">
+        <v>17</v>
+      </c>
+      <c r="G83" s="3" t="inlineStr">
+        <is>
+          <t>35m total (3m walk → 27m VTA Bus 57 North → VTA Orange Line East to Cisco Way → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H83" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I83" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J83" s="3">
+        <v>3231</v>
+      </c>
+      <c r="K83" s="3" t="inlineStr">
+        <is>
+          <t>825–910</t>
+        </is>
+      </c>
+      <c r="L83" s="3">
+        <v>0</v>
+      </c>
+      <c r="M83" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N83" s="3">
+        <v>215</v>
+      </c>
+      <c r="O83" s="3">
+        <v>3446</v>
+      </c>
+      <c r="P83" s="3">
+        <v>3446</v>
+      </c>
+      <c r="Q83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S83" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T83" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="U83" s="3" t="inlineStr">
+        <is>
+          <t>Greystar (Verified Market-Rate Luxury Community)</t>
+        </is>
+      </c>
+      <c r="V83" s="3" t="inlineStr">
+        <is>
+          <t>4.5★ resident rating! Huge 825–910 sq ft 1BR floor plans with $0 included garage parking, 4–6 weeks free, and instant I-280 access near Santana Row &amp; Mitsuwa.</t>
+        </is>
+      </c>
+      <c r="W83" s="3" t="inlineStr">
+        <is>
+          <t>Weekend guest parking fills up quickly; Saratoga Ave rush-hour traffic near I-280.</t>
+        </is>
+      </c>
+      <c r="X83" s="3" t="inlineStr">
+        <is>
+          <t>470 Saratoga Ave, San Jose, CA 95129</t>
+        </is>
+      </c>
+      <c r="Y83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/la-terraza-san-jose-ca/wucpje8/</t>
+        </is>
+      </c>
+      <c r="Z83" s="3" t="inlineStr">
+        <is>
+          <t>https://www.liveatlaterraza.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="42" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>Top Pick</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Avalon Willow Glen</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Midtown &amp; West SJ</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>4.2★ AvalonBay 1BR at $2,770 + Direct VTA Blue Line</t>
+        </is>
+      </c>
+      <c r="E84" s="3">
+        <v>11.3</v>
+      </c>
+      <c r="F84" s="3">
+        <v>18</v>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>37m total (5m walk → 27m VTA Blue Line → 5m walk)</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="J84" s="3">
+        <v>2770</v>
+      </c>
+      <c r="K84" s="3" t="inlineStr">
+        <is>
+          <t>726–814</t>
+        </is>
+      </c>
+      <c r="L84" s="3">
+        <v>0</v>
+      </c>
+      <c r="M84" s="3" t="inlineStr">
+        <is>
+          <t>PG&amp;E (~$0.44/kWh)</t>
+        </is>
+      </c>
+      <c r="N84" s="3">
+        <v>205</v>
+      </c>
+      <c r="O84" s="3">
+        <v>2975</v>
+      </c>
+      <c r="P84" s="3">
+        <v>2975</v>
+      </c>
+      <c r="Q84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S84" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T84" s="3">
+        <v>4.2</v>
+      </c>
+      <c r="U84" s="3" t="inlineStr">
+        <is>
+          <t>AvalonBay Communities (Verified Market-Rate Community (REIT))</t>
+        </is>
+      </c>
+      <c r="V84" s="3" t="inlineStr">
+        <is>
+          <t>4.2★ AvalonBay community where a spacious 726–814 sq ft 1BR starts at just $2,770/mo with $0 free parking AND walks directly to the VTA Blue Line (no transfers to Cisco Way!).</t>
+        </is>
+      </c>
+      <c r="W84" s="3" t="inlineStr">
+        <is>
+          <t>Garden walk-up buildings do not have elevators; unassigned surface spots fill up late at night.</t>
+        </is>
+      </c>
+      <c r="X84" s="3" t="inlineStr">
+        <is>
+          <t>3200 Rubino Dr, San Jose, CA 95125</t>
+        </is>
+      </c>
+      <c r="Y84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.apartments.com/avalon-willow-glen-san-jose-ca/4zfygh5/</t>
+        </is>
+      </c>
+      <c r="Z84" s="3" t="inlineStr">
+        <is>
+          <t>https://www.avaloncommunities.com/california/san-jose-apartments/avalon-willow-glen/</t>
         </is>
       </c>
     </row>

</xml_diff>